<commit_message>
Schedule: execute authorized TestRail sync (7 update + 2 add + 1 delete SCH-REAS-02)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/schedule-v1-testrail-import.xlsx
+++ b/testrail-import/schedule-v1-testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -6828,7 +6828,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>'Reassign' in the shift detail modal moves the shift to another technician</t>
+          <t>Right-click on any grid cell opens a context menu with New Shift, New Event, and View Day</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -6847,76 +6847,74 @@
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in on a desktop browser with Schedule: Edit.
-2. A shift exists on technician A; its detail modal is open.</t>
-        </is>
-      </c>
-      <c r="F131" s="2" t="inlineStr">
-        <is>
-          <t>1. Click the 'Reassign' action.
-2. Choose technician B and confirm.
-3. Check the grid and the line's roster.</t>
-        </is>
-      </c>
-      <c r="G131" s="2" t="inlineStr">
-        <is>
-          <t>1. The shift moves to technician B's row.
-2. The roster updates the same way as a drag reassignment (B added, A removed).
-3. A toast with Undo appears.</t>
-        </is>
-      </c>
-      <c r="H131" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §4.9 (Reassign action), §7</t>
-        </is>
-      </c>
-      <c r="I131" s="2" t="inlineStr"/>
-      <c r="J131" s="2" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" s="2" t="inlineStr">
-        <is>
-          <t>Right-click on any grid cell opens a context menu with New Shift, New Event, and View Day</t>
-        </is>
-      </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>Reassignment and Context Menu</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page in week view.</t>
         </is>
       </c>
-      <c r="F132" s="2" t="inlineStr">
+      <c r="F131" s="2" t="inlineStr">
         <is>
           <t>1. Right-click a technician's grid cell.
 2. Read the menu items.</t>
         </is>
       </c>
-      <c r="G132" s="2" t="inlineStr">
+      <c r="G131" s="2" t="inlineStr">
         <is>
           <t>1. A context menu opens at the cell.
 2. It contains: 'New Shift', 'New Event', and 'View Day'.
 3. The browser's own right-click menu does not appear instead.</t>
         </is>
       </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md §7 (Right-click context menu)</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr"/>
+      <c r="J131" s="2" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>'View Day' in the context menu opens day view for that cell's date</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Reassignment and Context Menu</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in on a desktop browser with Schedule: Edit.
+2. You are on the Schedule page in week or month view.</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>1. Right-click a cell on a specific day.
+2. Choose 'View Day'.</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>1. The grid switches to day view showing that cell's date.
+2. The toolbar date label and the Day/Week/Month control reflect the switch.</t>
+        </is>
+      </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Right-click context menu)</t>
+          <t>requirements.md §7 (Right-click context menu - View Day)</t>
         </is>
       </c>
       <c r="I132" s="2" t="inlineStr"/>
@@ -6925,7 +6923,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>'View Day' in the context menu opens day view for that cell's date</t>
+          <t>'New Shift' in the context menu starts shift creation for that technician and day</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -6944,164 +6942,117 @@
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in on a desktop browser with Schedule: Edit.
-2. You are on the Schedule page in week or month view.</t>
-        </is>
-      </c>
-      <c r="F133" s="2" t="inlineStr">
-        <is>
-          <t>1. Right-click a cell on a specific day.
-2. Choose 'View Day'.</t>
-        </is>
-      </c>
-      <c r="G133" s="2" t="inlineStr">
-        <is>
-          <t>1. The grid switches to day view showing that cell's date.
-2. The toolbar date label and the Day/Week/Month control reflect the switch.</t>
-        </is>
-      </c>
-      <c r="H133" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Right-click context menu - View Day)</t>
-        </is>
-      </c>
-      <c r="I133" s="2" t="inlineStr"/>
-      <c r="J133" s="2" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="inlineStr">
-        <is>
-          <t>'New Shift' in the context menu starts shift creation for that technician and day</t>
-        </is>
-      </c>
-      <c r="B134" s="2" t="inlineStr">
-        <is>
-          <t>Reassignment and Context Menu</t>
-        </is>
-      </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E134" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. Schedulable work order lines exist.
 3. You are on the Schedule page in week view.</t>
         </is>
       </c>
-      <c r="F134" s="2" t="inlineStr">
+      <c r="F133" s="2" t="inlineStr">
         <is>
           <t>1. Right-click a technician's cell and choose 'New Shift'.
 2. Complete the creation flow that opens.</t>
         </is>
       </c>
-      <c r="G134" s="2" t="inlineStr">
+      <c r="G133" s="2" t="inlineStr">
         <is>
           <t>1. A shift-creation flow opens targeted at that technician and day.
 2. Completing it creates a shift in that cell, following the same scope/spread rules as drag-and-drop.</t>
         </is>
       </c>
-      <c r="H134" s="2" t="inlineStr">
+      <c r="H133" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (Right-click context menu - New Shift), §14.1 (creation via context menu)</t>
         </is>
       </c>
-      <c r="I134" s="2" t="inlineStr"/>
-      <c r="J134" s="2" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="inlineStr">
+      <c r="I133" s="2" t="inlineStr"/>
+      <c r="J133" s="2" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
         <is>
           <t>Deleting a middle shift of a series asks for scope with all three options, each stating the hours returned</t>
         </is>
       </c>
-      <c r="B135" s="2" t="inlineStr">
+      <c r="B134" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C135" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D135" s="2" t="inlineStr">
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E135" s="2" t="inlineStr">
+      <c r="E134" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 3 shifts exists for one technician.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F135" s="2" t="inlineStr">
+      <c r="F134" s="2" t="inlineStr">
         <is>
           <t>1. Delete a MIDDLE shift of the series (via the detail modal's Delete).
 2. Read the scope options offered (do not confirm yet).</t>
         </is>
       </c>
-      <c r="G135" s="2" t="inlineStr">
+      <c r="G134" s="2" t="inlineStr">
         <is>
           <t>1. A scope prompt appears with three options: this shift only, this and everything after, and the whole series.
 2. Each option states its consequence in hours returned (spec's example format: 'returns 8h' / 'returns 56h').
 3. The prompt uses routine, lightweight styling - not alarming destructive styling.</t>
         </is>
       </c>
-      <c r="H135" s="2" t="inlineStr">
+      <c r="H134" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (Series-aware deletion)</t>
         </is>
       </c>
-      <c r="I135" s="2" t="inlineStr"/>
-      <c r="J135" s="2" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="inlineStr">
+      <c r="I134" s="2" t="inlineStr"/>
+      <c r="J134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
         <is>
           <t>'This shift only' removes that day, the series keeps the gap, and the hours return to the estimate's remaining</t>
         </is>
       </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B135" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E136" s="2" t="inlineStr">
+      <c r="E135" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 3 shifts exists; note the total scheduled hours.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F136" s="2" t="inlineStr">
+      <c r="F135" s="2" t="inlineStr">
         <is>
           <t>1. Delete a middle shift with the 'this shift only' scope.
 2. Look at the series on the grid.
 3. Check the scheduled hours.</t>
         </is>
       </c>
-      <c r="G136" s="2" t="inlineStr">
+      <c r="G135" s="2" t="inlineStr">
         <is>
           <t>1. Only that day's shift is removed.
 2. The series keeps the gap - the remaining shifts do NOT shuffle to close it.
@@ -7109,148 +7060,148 @@
 4. An undo toast appears.</t>
         </is>
       </c>
-      <c r="H136" s="2" t="inlineStr">
+      <c r="H135" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (This shift only)</t>
         </is>
       </c>
-      <c r="I136" s="2" t="inlineStr"/>
-      <c r="J136" s="2" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="inlineStr">
+      <c r="I135" s="2" t="inlineStr"/>
+      <c r="J135" s="2" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
         <is>
           <t>'This and everything after' removes from the clicked shift onward, keeping earlier shifts</t>
         </is>
       </c>
-      <c r="B137" s="2" t="inlineStr">
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C137" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D137" s="2" t="inlineStr">
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E137" s="2" t="inlineStr">
+      <c r="E136" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 4 shifts exists.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F137" s="2" t="inlineStr">
+      <c r="F136" s="2" t="inlineStr">
         <is>
           <t>1. Delete the series' THIRD shift with the 'this and everything after' scope.
 2. Look at the series on the grid.</t>
         </is>
       </c>
-      <c r="G137" s="2" t="inlineStr">
+      <c r="G136" s="2" t="inlineStr">
         <is>
           <t>1. The third shift and every later shift of the series are removed.
 2. The first two shifts remain untouched.
 3. An undo toast appears.</t>
         </is>
       </c>
-      <c r="H137" s="2" t="inlineStr">
+      <c r="H136" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (This and everything after)</t>
         </is>
       </c>
-      <c r="I137" s="2" t="inlineStr"/>
-      <c r="J137" s="2" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
+      <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
         <is>
           <t>'The whole series' removes all of the series' shifts for that technician</t>
         </is>
       </c>
-      <c r="B138" s="2" t="inlineStr">
+      <c r="B137" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E138" s="2" t="inlineStr">
+      <c r="E137" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. The SAME work order has a series on technician A and an independent series on technician B.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F138" s="2" t="inlineStr">
+      <c r="F137" s="2" t="inlineStr">
         <is>
           <t>1. Delete one of technician A's series shifts with the 'whole series' scope.
 2. Look at both technicians' rows.</t>
         </is>
       </c>
-      <c r="G138" s="2" t="inlineStr">
+      <c r="G137" s="2" t="inlineStr">
         <is>
           <t>1. All of technician A's series shifts are removed.
 2. Technician B's independent series is untouched (the scope is per technician's series).
 3. An undo toast appears.</t>
         </is>
       </c>
-      <c r="H138" s="2" t="inlineStr">
+      <c r="H137" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (The whole series - 'for that technician')</t>
         </is>
       </c>
-      <c r="I138" s="2" t="inlineStr"/>
-      <c r="J138" s="2" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="inlineStr">
+      <c r="I137" s="2" t="inlineStr"/>
+      <c r="J137" s="2" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
         <is>
           <t>Scope options adapt to position: first and last shifts of a series each show only two options</t>
         </is>
       </c>
-      <c r="B139" s="2" t="inlineStr">
+      <c r="B138" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C139" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D139" s="2" t="inlineStr">
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E139" s="2" t="inlineStr">
+      <c r="E138" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 3 shifts exists.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr">
+      <c r="F138" s="2" t="inlineStr">
         <is>
           <t>1. Start deleting the FIRST shift of the series; read the options, then cancel.
 2. Start deleting the LAST shift; read the options, then cancel.
 3. Start deleting a MIDDLE shift; read the options, then cancel.</t>
         </is>
       </c>
-      <c r="G139" s="2" t="inlineStr">
+      <c r="G138" s="2" t="inlineStr">
         <is>
           <t>1. First shift: two options ('this and after' would equal 'whole series', so only two are shown).
 2. Last shift: two options ('this and after' would equal 'this only').
@@ -7258,91 +7209,91 @@
 4. Cancelling leaves the series unchanged in every case.</t>
         </is>
       </c>
-      <c r="H139" s="2" t="inlineStr">
+      <c r="H138" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (options adapt to position)</t>
         </is>
       </c>
-      <c r="I139" s="2" t="inlineStr"/>
-      <c r="J139" s="2" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
+      <c r="I138" s="2" t="inlineStr"/>
+      <c r="J138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
         <is>
           <t>Deleting a standalone (non-series) shift does not ask for a series scope</t>
         </is>
       </c>
-      <c r="B140" s="2" t="inlineStr">
+      <c r="B139" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E140" s="2" t="inlineStr">
+      <c r="E139" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A single standalone shift (not part of any series) exists.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr">
+      <c r="F139" s="2" t="inlineStr">
         <is>
           <t>1. Delete the standalone shift.
 2. Watch what is asked.</t>
         </is>
       </c>
-      <c r="G140" s="2" t="inlineStr">
+      <c r="G139" s="2" t="inlineStr">
         <is>
           <t>1. No series-scope prompt appears (the scope question is only for shifts that belong to a series).
 2. The shift is deleted and an undo toast appears.</t>
         </is>
       </c>
-      <c r="H140" s="2" t="inlineStr">
+      <c r="H139" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (derived - scope prompt is for series shifts)</t>
         </is>
       </c>
-      <c r="I140" s="2" t="inlineStr"/>
-      <c r="J140" s="2" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
+      <c r="I139" s="2" t="inlineStr"/>
+      <c r="J139" s="2" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
         <is>
           <t>Every create, delete, move, and reassign action produces a toast with an Undo option</t>
         </is>
       </c>
-      <c r="B141" s="2" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C141" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E141" s="2" t="inlineStr">
+      <c r="E140" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. Schedulable lines and an existing shift are available.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F141" s="2" t="inlineStr">
+      <c r="F140" s="2" t="inlineStr">
         <is>
           <t>1. Create a shift - watch for a toast.
 2. Move a shift to another day - watch for a toast.
@@ -7350,98 +7301,98 @@
 4. Delete a shift - watch for a toast.</t>
         </is>
       </c>
-      <c r="G141" s="2" t="inlineStr">
+      <c r="G140" s="2" t="inlineStr">
         <is>
           <t>1. Each of the four actions produces a toast notification.
 2. Every toast offers an Undo option.</t>
         </is>
       </c>
-      <c r="H141" s="2" t="inlineStr">
+      <c r="H140" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (Toast notifications), §11 (Undo)</t>
         </is>
       </c>
-      <c r="I141" s="2" t="inlineStr"/>
-      <c r="J141" s="2" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
+      <c r="I140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
         <is>
           <t>The toast persists 4 to 7 seconds, stays while the cursor is over it, and dismisses on mouse-leave</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="B141" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E142" s="2" t="inlineStr">
+      <c r="E141" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
+      <c r="F141" s="2" t="inlineStr">
         <is>
           <t>1. Perform an action that shows a toast (for example move a shift) and let the toast sit untouched - time how long it stays.
 2. Trigger another toast and hold the cursor OVER it well past its normal lifetime.
 3. Move the cursor off the toast.</t>
         </is>
       </c>
-      <c r="G142" s="2" t="inlineStr">
+      <c r="G141" s="2" t="inlineStr">
         <is>
           <t>1. Untouched, the toast persists for roughly 4 to 7 seconds before dismissing.
 2. While the cursor is over it, the toast stays (does not auto-dismiss).
 3. After the cursor leaves, it dismisses.</t>
         </is>
       </c>
-      <c r="H142" s="2" t="inlineStr">
+      <c r="H141" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (Toast notifications), §11 (Undo)</t>
         </is>
       </c>
-      <c r="I142" s="2" t="inlineStr"/>
-      <c r="J142" s="2" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="2" t="inlineStr">
+      <c r="I141" s="2" t="inlineStr"/>
+      <c r="J141" s="2" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
         <is>
           <t>Undo restores the state before the action - for delete, move, and reassign</t>
         </is>
       </c>
-      <c r="B143" s="2" t="inlineStr">
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D143" s="2" t="inlineStr">
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E143" s="2" t="inlineStr">
+      <c r="E142" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A shift exists; note its technician, day, and time.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr">
+      <c r="F142" s="2" t="inlineStr">
         <is>
           <t>1. Delete the shift, then click Undo on the toast.
 2. Move the shift to another day, then click Undo.
@@ -7449,7 +7400,7 @@
 4. Check the line's roster after the reassign undo.</t>
         </is>
       </c>
-      <c r="G143" s="2" t="inlineStr">
+      <c r="G142" s="2" t="inlineStr">
         <is>
           <t>1. Undo after delete: the shift is back exactly where it was.
 2. Undo after move: the shift returns to its original day/time.
@@ -7457,91 +7408,91 @@
 4. Every destructive action is undoable within the toast's lifetime.</t>
         </is>
       </c>
-      <c r="H143" s="2" t="inlineStr">
+      <c r="H142" s="2" t="inlineStr">
         <is>
           <t>requirements.md §11 (Undo), §7</t>
         </is>
       </c>
-      <c r="I143" s="2" t="inlineStr"/>
-      <c r="J143" s="2" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="inlineStr">
+      <c r="I142" s="2" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
         <is>
           <t>Escape closes the topmost open modal or popover, following the stacking order</t>
         </is>
       </c>
-      <c r="B144" s="2" t="inlineStr">
+      <c r="B143" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E144" s="2" t="inlineStr">
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr">
+      <c r="F143" s="2" t="inlineStr">
         <is>
           <t>1. Open the shift detail modal, then open a popover on top of it (for example the color picker or a filter/search popover elsewhere).
 2. Press Escape once.
 3. Press Escape again.</t>
         </is>
       </c>
-      <c r="G144" s="2" t="inlineStr">
+      <c r="G143" s="2" t="inlineStr">
         <is>
           <t>1. The FIRST Escape closes only the topmost layer (the popover), leaving the layer beneath open.
 2. The SECOND Escape closes the next layer down.
 3. Escape works anywhere on the schedule page as a global shortcut, following the defined stacking order (delete scope, reassign, spread, capacity, event modal, event view, line picker, shift detail, cell menu, calendar picker, customize, filters, search).</t>
         </is>
       </c>
-      <c r="H144" s="2" t="inlineStr">
+      <c r="H143" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (Keyboard support - Escape)</t>
         </is>
       </c>
-      <c r="I144" s="2" t="inlineStr"/>
-      <c r="J144" s="2" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="inlineStr">
+      <c r="I143" s="2" t="inlineStr"/>
+      <c r="J143" s="2" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
         <is>
           <t>Within the shift modal, Escape first dismisses an open sub-picker before closing the modal itself</t>
         </is>
       </c>
-      <c r="B145" s="2" t="inlineStr">
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C145" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D145" s="2" t="inlineStr">
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E145" s="2" t="inlineStr">
+      <c r="E144" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's detail modal is open.</t>
         </is>
       </c>
-      <c r="F145" s="2" t="inlineStr">
+      <c r="F144" s="2" t="inlineStr">
         <is>
           <t>1. Open the color picker inside the modal, press Escape, and watch.
 2. Open the time picker, press Escape.
@@ -7549,50 +7500,50 @@
 4. With nothing open inside the modal, press Escape.</t>
         </is>
       </c>
-      <c r="G145" s="2" t="inlineStr">
+      <c r="G144" s="2" t="inlineStr">
         <is>
           <t>1. Escape with the color picker open closes only the color picker - the modal stays open.
 2. Same for the time picker and the note edit.
 3. Escape with no open sub-picker closes the modal itself.</t>
         </is>
       </c>
-      <c r="H145" s="2" t="inlineStr">
+      <c r="H144" s="2" t="inlineStr">
         <is>
           <t>requirements.md §7 (Escape within the shift modal)</t>
         </is>
       </c>
-      <c r="I145" s="2" t="inlineStr"/>
-      <c r="J145" s="2" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="inlineStr">
+      <c r="I144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
         <is>
           <t>Enter confirms the active confirmable dialog (delete scope, reassign, spread, event create/edit)</t>
         </is>
       </c>
-      <c r="B146" s="2" t="inlineStr">
+      <c r="B145" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C146" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D146" s="2" t="inlineStr">
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E146" s="2" t="inlineStr">
+      <c r="E145" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. Shifts/series and events exist to exercise the dialogs.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F146" s="2" t="inlineStr">
+      <c r="F145" s="2" t="inlineStr">
         <is>
           <t>1. Open the spread step for a large job, press Enter.
 2. Open the reassign dialog for a shift, choose a technician, press Enter.
@@ -7600,15 +7551,62 @@
 4. Open a series delete-scope prompt, select a scope, press Enter.</t>
         </is>
       </c>
-      <c r="G146" s="2" t="inlineStr">
+      <c r="G145" s="2" t="inlineStr">
         <is>
           <t>1. In each confirmable dialog, Enter confirms it - equivalent to clicking its confirm action.
 2. The confirmed action takes effect (spread created / reassigned / event saved / delete applied).</t>
         </is>
       </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md §7 (Keyboard support - Enter)</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr"/>
+      <c r="J145" s="2" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>Enter does not fire inside textareas - multiline note editing works normally</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Keyboard Interactions</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in on a desktop browser with Schedule: Edit.
+2. A shift's detail modal is open with the note editor active.</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>1. Type a line of note text and press Enter.
+2. Type a second line.</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>1. Enter inserts a new line in the note - it does NOT confirm/close the dialog.
+2. The multiline note can be completed and saved normally.</t>
+        </is>
+      </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Keyboard support - Enter)</t>
+          <t>requirements.md §7 (Enter does not fire inside textareas)</t>
         </is>
       </c>
       <c r="I146" s="2" t="inlineStr"/>
@@ -7617,7 +7615,7 @@
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>Enter does not fire inside textareas - multiline note editing works normally</t>
+          <t>Modals trap focus and all interactive elements are keyboard-reachable</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -7627,7 +7625,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -7636,205 +7634,158 @@
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in on a desktop browser with Schedule: Edit.
-2. A shift's detail modal is open with the note editor active.</t>
-        </is>
-      </c>
-      <c r="F147" s="2" t="inlineStr">
-        <is>
-          <t>1. Type a line of note text and press Enter.
-2. Type a second line.</t>
-        </is>
-      </c>
-      <c r="G147" s="2" t="inlineStr">
-        <is>
-          <t>1. Enter inserts a new line in the note - it does NOT confirm/close the dialog.
-2. The multiline note can be completed and saved normally.</t>
-        </is>
-      </c>
-      <c r="H147" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Enter does not fire inside textareas)</t>
-        </is>
-      </c>
-      <c r="I147" s="2" t="inlineStr"/>
-      <c r="J147" s="2" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="inlineStr">
-        <is>
-          <t>Modals trap focus and all interactive elements are keyboard-reachable</t>
-        </is>
-      </c>
-      <c r="B148" s="2" t="inlineStr">
-        <is>
-          <t>Keyboard Interactions</t>
-        </is>
-      </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>Accessibility</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's detail modal is open.</t>
         </is>
       </c>
-      <c r="F148" s="2" t="inlineStr">
+      <c r="F147" s="2" t="inlineStr">
         <is>
           <t>1. Press Tab repeatedly and watch where focus goes.
 2. Continue tabbing past the last control in the modal.
 3. Close the modal and Tab through the schedule page's toolbar and sidebar controls.</t>
         </is>
       </c>
-      <c r="G148" s="2" t="inlineStr">
+      <c r="G147" s="2" t="inlineStr">
         <is>
           <t>1. Focus moves through the modal's interactive elements with visible focus rings.
 2. Focus stays trapped inside the modal (wraps back to its first control) until the modal closes.
 3. On the page, toolbar and sidebar controls are reachable by keyboard.</t>
         </is>
       </c>
-      <c r="H148" s="2" t="inlineStr">
+      <c r="H147" s="2" t="inlineStr">
         <is>
           <t>requirements.md §11 (Accessibility)</t>
         </is>
       </c>
-      <c r="I148" s="2" t="inlineStr"/>
-      <c r="J148" s="2" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="I147" s="2" t="inlineStr"/>
+      <c r="J147" s="2" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
         <is>
           <t>Blue is the default color for all shifts, including long and multi-week jobs</t>
         </is>
       </c>
-      <c r="B149" s="2" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>Color System</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="inlineStr">
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E149" s="2" t="inlineStr">
+      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F149" s="2" t="inlineStr">
+      <c r="F148" s="2" t="inlineStr">
         <is>
           <t>1. Create a normal single-day shift without touching any color option.
 2. Create a multi-week series without touching any color option.
 3. Look at both on the grid.</t>
         </is>
       </c>
-      <c r="G149" s="2" t="inlineStr">
+      <c r="G148" s="2" t="inlineStr">
         <is>
           <t>1. Both the single shift and the multi-week series render in the default blue.
 2. No special color is auto-applied to long jobs - blue is the default for ALL shifts.</t>
         </is>
       </c>
-      <c r="H149" s="2" t="inlineStr">
+      <c r="H148" s="2" t="inlineStr">
         <is>
           <t>requirements.md §10</t>
         </is>
       </c>
-      <c r="I149" s="2" t="inlineStr"/>
-      <c r="J149" s="2" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+      <c r="I148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
         <is>
           <t>Choosing a color from the shift modal's picker recolors the shift with matching background, text, and accent tones</t>
         </is>
       </c>
-      <c r="B150" s="2" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>Color System</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E150" s="2" t="inlineStr">
+      <c r="E149" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift exists; its detail modal is open.</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr">
+      <c r="F149" s="2" t="inlineStr">
         <is>
           <t>1. Open the color picker in the modal.
 2. Choose a non-default color.
 3. Look at the block on the grid.</t>
         </is>
       </c>
-      <c r="G150" s="2" t="inlineStr">
+      <c r="G149" s="2" t="inlineStr">
         <is>
           <t>1. The shift's block re-renders in the chosen color.
 2. The color provides three consistent tones: background fill, text color, and accent (left border).
 3. Colors carry no fixed meaning - they are free choice beyond the two defaults (blue shift / grey event).</t>
         </is>
       </c>
-      <c r="H150" s="2" t="inlineStr">
+      <c r="H149" s="2" t="inlineStr">
         <is>
           <t>requirements.md §10, §4.9 (Color picker)</t>
         </is>
       </c>
-      <c r="I150" s="2" t="inlineStr"/>
-      <c r="J150" s="2" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
+      <c r="I149" s="2" t="inlineStr"/>
+      <c r="J149" s="2" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
         <is>
           <t>Color labels are editable per shop</t>
         </is>
       </c>
-      <c r="B151" s="2" t="inlineStr">
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>Color System</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E151" s="2" t="inlineStr">
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's or event's color picker is open.</t>
         </is>
       </c>
-      <c r="F151" s="2" t="inlineStr">
+      <c r="F150" s="2" t="inlineStr">
         <is>
           <t>1. Find the editable label of one color in the picker.
 2. Rename it (for example to 'ZZAUTOTEST Rush').
@@ -7842,50 +7793,50 @@
 4. Restore the original label.</t>
         </is>
       </c>
-      <c r="G151" s="2" t="inlineStr">
+      <c r="G150" s="2" t="inlineStr">
         <is>
           <t>1. Each color's label can be edited.
 2. The renamed label shows for the whole shop - the same picker opened elsewhere shows 'ZZAUTOTEST Rush'.
 3. Shifts and events share the same custom palette with the same labels.</t>
         </is>
       </c>
-      <c r="H151" s="2" t="inlineStr">
+      <c r="H150" s="2" t="inlineStr">
         <is>
           <t>requirements.md §10 (Color labels are editable per shop), §4.10 (shared picker)</t>
         </is>
       </c>
-      <c r="I151" s="2" t="inlineStr"/>
-      <c r="J151" s="2" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
+      <c r="I150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
         <is>
           <t>Schedule: View grants the full read experience - page, all three views, mini calendar, search, filter, tooltips, read-only modals</t>
         </is>
       </c>
-      <c r="B152" s="2" t="inlineStr">
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C152" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D152" s="2" t="inlineStr">
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E152" s="2" t="inlineStr">
+      <c r="E151" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: View but NOT Edit (assign a suitable system role or a purpose-made custom role; restore after).
 2. Shifts and events exist on the grid, created by an Edit-capable user.
 3. You are signed in AS that View-only user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F152" s="2" t="inlineStr">
+      <c r="F151" s="2" t="inlineStr">
         <is>
           <t>1. Open the Schedule page.
 2. Switch between Day, Week, and Month.
@@ -7893,7 +7844,7 @@
 4. Hover a shift for its tooltip, then click it to open the detail modal.</t>
         </is>
       </c>
-      <c r="G152" s="2" t="inlineStr">
+      <c r="G151" s="2" t="inlineStr">
         <is>
           <t>1. The Schedule page opens and all three views work.
 2. The mini calendar, search, and filters all work.
@@ -7901,43 +7852,43 @@
 4. Tooltips show on hover, and the shift/event detail modals open in read-only mode.</t>
         </is>
       </c>
-      <c r="H152" s="2" t="inlineStr">
+      <c r="H151" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.1 (Schedule: View), §14.3</t>
         </is>
       </c>
-      <c r="I152" s="2" t="inlineStr"/>
-      <c r="J152" s="2" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
+      <c r="I151" s="2" t="inlineStr"/>
+      <c r="J151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t>View-only: every editing affordance is hidden or disabled</t>
         </is>
       </c>
-      <c r="B153" s="2" t="inlineStr">
+      <c r="B152" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C153" s="2" t="inlineStr">
+      <c r="C152" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E153" s="2" t="inlineStr">
+      <c r="E152" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: View but NOT Edit.
 2. Shifts, a series, and events exist on the grid.
 3. You are signed in AS that View-only user on a desktop browser, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F153" s="2" t="inlineStr">
+      <c r="F152" s="2" t="inlineStr">
         <is>
           <t>1. Look for drag handles on sidebar lines and try to drag a work order card onto the grid.
 2. Try dragging an existing shift block (move/reassign) and look for resize handles in day view.
@@ -7945,7 +7896,7 @@
 4. Open a shift's detail modal and inspect its fields and actions.</t>
         </is>
       </c>
-      <c r="G153" s="2" t="inlineStr">
+      <c r="G152" s="2" t="inlineStr">
         <is>
           <t>1. No drag handles are offered and nothing can be dragged from the sidebar onto the grid.
 2. Shift blocks cannot be moved or resized - no drop targets or resize handles appear.
@@ -7953,9 +7904,56 @@
 4. In the modal, edit fields are hidden or disabled, and the reassign and delete actions are absent.</t>
         </is>
       </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md §14.1 (Schedule: View - editing affordances hidden or disabled)</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>With Schedule: View OFF, the Schedule top-level nav item is hidden entirely</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>1. A test user's role has Schedule: View OFF (no Schedule permission).
+2. You are signed in AS that user on a desktop browser.</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>1. Look at the app's main navigation.
+2. Search the nav for any Schedule entry.</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>1. The Schedule top-level nav item is not shown at all.
+2. The rest of the app works normally for the role.</t>
+        </is>
+      </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §14.1 (Schedule: View - editing affordances hidden or disabled)</t>
+          <t>requirements.md §14.1 (When Schedule: View is OFF)</t>
         </is>
       </c>
       <c r="I153" s="2" t="inlineStr"/>
@@ -7964,7 +7962,7 @@
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>With Schedule: View OFF, the Schedule top-level nav item is hidden entirely</t>
+          <t>Schedule: Edit unlocks all creation and modification interactions</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -7974,7 +7972,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -7983,59 +7981,12 @@
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
-        <is>
-          <t>1. A test user's role has Schedule: View OFF (no Schedule permission).
-2. You are signed in AS that user on a desktop browser.</t>
-        </is>
-      </c>
-      <c r="F154" s="2" t="inlineStr">
-        <is>
-          <t>1. Look at the app's main navigation.
-2. Search the nav for any Schedule entry.</t>
-        </is>
-      </c>
-      <c r="G154" s="2" t="inlineStr">
-        <is>
-          <t>1. The Schedule top-level nav item is not shown at all.
-2. The rest of the app works normally for the role.</t>
-        </is>
-      </c>
-      <c r="H154" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (When Schedule: View is OFF)</t>
-        </is>
-      </c>
-      <c r="I154" s="2" t="inlineStr"/>
-      <c r="J154" s="2" t="inlineStr"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
-        <is>
-          <t>Schedule: Edit unlocks all creation and modification interactions</t>
-        </is>
-      </c>
-      <c r="B155" s="2" t="inlineStr">
-        <is>
-          <t>Permissions</t>
-        </is>
-      </c>
-      <c r="C155" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D155" s="2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="E155" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: Edit (and View) but NOT Delete.
 2. Work orders with approved lines exist; you are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F155" s="2" t="inlineStr">
+      <c r="F154" s="2" t="inlineStr">
         <is>
           <t>1. Drag a work order from the sidebar onto a technician cell and complete the scope picker (and spread modal for a large job).
 2. Right-click a cell and create an event via 'New Event'; in day view, click empty space to create.
@@ -8044,7 +7995,7 @@
 5. Edit fields in the shift and event detail modals.</t>
         </is>
       </c>
-      <c r="G155" s="2" t="inlineStr">
+      <c r="G154" s="2" t="inlineStr">
         <is>
           <t>1. Drag-and-drop from the sidebar, the scope picker, and the spread modal all work.
 2. Shift and event creation works, including via the right-click context menu and day-view click-to-create.
@@ -8053,100 +8004,100 @@
 5. Modal fields are editable and save.</t>
         </is>
       </c>
-      <c r="H155" s="2" t="inlineStr">
+      <c r="H154" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.1 (Schedule: Edit)</t>
         </is>
       </c>
-      <c r="I155" s="2" t="inlineStr"/>
-      <c r="J155" s="2" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="inlineStr">
+      <c r="I154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>Edit without Delete: the user can create and modify but cannot remove - delete action and trash icon hidden</t>
         </is>
       </c>
-      <c r="B156" s="2" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C156" s="2" t="inlineStr">
+      <c r="C155" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D156" s="2" t="inlineStr">
+      <c r="D155" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E156" s="2" t="inlineStr">
+      <c r="E155" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: Edit but NOT Delete.
 2. A shift, a series, and an event exist (some created by this user).
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F156" s="2" t="inlineStr">
+      <c r="F155" s="2" t="inlineStr">
         <is>
           <t>1. Open a shift's detail modal and look for the delete action / trash icon.
 2. Open an event's modal and look for a delete action.
 3. Try to find ANY way to remove a shift or event.</t>
         </is>
       </c>
-      <c r="G156" s="2" t="inlineStr">
+      <c r="G155" s="2" t="inlineStr">
         <is>
           <t>1. The delete action and the trash icon are hidden in the shift modal.
 2. Events likewise offer no delete.
 3. No path exists to remove shifts or events - while creating and modifying still work.</t>
         </is>
       </c>
-      <c r="H156" s="2" t="inlineStr">
+      <c r="H155" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.1 (Schedule: Delete - without it)</t>
         </is>
       </c>
-      <c r="I156" s="2" t="inlineStr"/>
-      <c r="J156" s="2" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="inlineStr">
+      <c r="I155" s="2" t="inlineStr"/>
+      <c r="J155" s="2" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
         <is>
           <t>Schedule: Delete unlocks deleting shifts and events, including the three series-aware scopes</t>
         </is>
       </c>
-      <c r="B157" s="2" t="inlineStr">
+      <c r="B156" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C157" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D157" s="2" t="inlineStr">
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E157" s="2" t="inlineStr">
+      <c r="E156" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: Delete.
 2. A standalone shift, a series, and an event exist.
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F157" s="2" t="inlineStr">
+      <c r="F156" s="2" t="inlineStr">
         <is>
           <t>1. Delete the standalone shift.
 2. Delete a series shift and read the scope options.
 3. Delete the event.</t>
         </is>
       </c>
-      <c r="G157" s="2" t="inlineStr">
+      <c r="G156" s="2" t="inlineStr">
         <is>
           <t>1. The delete action is available and works for shifts.
 2. Series deletion offers its scopes (this shift / this and after / whole series).
@@ -8154,204 +8105,251 @@
 4. Undo toasts appear (restore the items via Undo to clean up).</t>
         </is>
       </c>
-      <c r="H157" s="2" t="inlineStr">
+      <c r="H156" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.1 (Schedule: Delete)</t>
         </is>
       </c>
-      <c r="I157" s="2" t="inlineStr"/>
-      <c r="J157" s="2" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="inlineStr">
+      <c r="I156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
         <is>
           <t>The permission tiers depend on each other: Delete requires Edit, and Edit requires View</t>
         </is>
       </c>
-      <c r="B158" s="2" t="inlineStr">
+      <c r="B157" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C158" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D158" s="2" t="inlineStr">
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E158" s="2" t="inlineStr">
+      <c r="E157" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as an admin who can edit custom roles.
 2. A ZZAUTOTEST custom role exists (create one; delete after).</t>
         </is>
       </c>
-      <c r="F158" s="2" t="inlineStr">
+      <c r="F157" s="2" t="inlineStr">
         <is>
           <t>1. In the role's Schedule permissions, try to enable Edit while View is off.
 2. Try to enable Delete while Edit is off.
 3. Enable View, then Edit, then Delete in order.</t>
         </is>
       </c>
-      <c r="G158" s="2" t="inlineStr">
+      <c r="G157" s="2" t="inlineStr">
         <is>
           <t>1. Edit cannot be granted without View (the admin UI enforces or auto-selects the dependency).
 2. Delete cannot be granted without Edit.
 3. The three tiers can be enabled in dependency order, so each higher level always includes the ones beneath it (Delete includes Edit, and Edit includes View).</t>
         </is>
       </c>
-      <c r="H158" s="2" t="inlineStr">
+      <c r="H157" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14 (Delete requires Edit and Edit requires View)</t>
         </is>
       </c>
-      <c r="I158" s="2" t="inlineStr"/>
-      <c r="J158" s="2" t="inlineStr"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
+      <c r="I157" s="2" t="inlineStr"/>
+      <c r="J157" s="2" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
         <is>
           <t>Schedule access without Work Orders: View - sidebar hides the WO list and drill-down; mini calendar stays; grid shifts remain usable</t>
         </is>
       </c>
-      <c r="B159" s="2" t="inlineStr">
+      <c r="B158" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C159" s="2" t="inlineStr">
+      <c r="C158" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D159" s="2" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E159" s="2" t="inlineStr">
+      <c r="E158" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule access but Work Orders: View OFF.
 2. Shifts already exist on the grid.
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F159" s="2" t="inlineStr">
+      <c r="F158" s="2" t="inlineStr">
         <is>
           <t>1. Look at the left sidebar.
 2. Interact with the shifts already on the grid (hover, open modal, and - if the role has Edit - move one).
 3. Try to find any way to drag a new work order onto the grid.</t>
         </is>
       </c>
-      <c r="G159" s="2" t="inlineStr">
+      <c r="G158" s="2" t="inlineStr">
         <is>
           <t>1. The sidebar hides the work order list and the line drill-down; the mini calendar remains available.
 2. Shifts already on the grid can still be viewed and interacted with per the role's Schedule tier.
 3. New work orders cannot be dragged on - the WO list is simply not visible.</t>
         </is>
       </c>
-      <c r="H159" s="2" t="inlineStr">
+      <c r="H158" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.2</t>
         </is>
       </c>
-      <c r="I159" s="2" t="inlineStr"/>
-      <c r="J159" s="2" t="inlineStr"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="inlineStr">
+      <c r="I158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
         <is>
           <t>No own-only restriction: every Schedule: View user sees ALL technicians' shifts and events</t>
         </is>
       </c>
-      <c r="B160" s="2" t="inlineStr">
+      <c r="B159" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="inlineStr">
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E160" s="2" t="inlineStr">
+      <c r="E159" s="2" t="inlineStr">
         <is>
           <t>1. Shifts and events exist for SEVERAL different technicians.
 2. A test user with a low-tier View-only role exists (and is themselves one of the technicians).
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F160" s="2" t="inlineStr">
+      <c r="F159" s="2" t="inlineStr">
         <is>
           <t>1. Read the grid across all departments and technicians.
 2. Check 'My Shifts' in 'Filter and Display' is OFF (default).</t>
         </is>
       </c>
-      <c r="G160" s="2" t="inlineStr">
+      <c r="G159" s="2" t="inlineStr">
         <is>
           <t>1. The user sees ALL technicians' shifts and events, not only their own - there is no role-based 'own shifts only' restriction.
 2. 'My Shifts' exists only as an optional personal convenience filter (off by default), not a security boundary.</t>
         </is>
       </c>
-      <c r="H160" s="2" t="inlineStr">
+      <c r="H159" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.3</t>
         </is>
       </c>
-      <c r="I160" s="2" t="inlineStr"/>
-      <c r="J160" s="2" t="inlineStr"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="inlineStr">
+      <c r="I159" s="2" t="inlineStr"/>
+      <c r="J159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
         <is>
           <t>Grid rows are department-based: any staff member in a visible department appears as a row, regardless of role</t>
         </is>
       </c>
-      <c r="B161" s="2" t="inlineStr">
+      <c r="B160" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C161" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D161" s="2" t="inlineStr">
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E161" s="2" t="inlineStr">
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>1. A staff member with a NON-technician role (for example Office) is assigned to a department that is visible on the schedule (set up; restore after).
 2. Another staff member has NO department assignment.
 3. You are signed in on a desktop browser, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F161" s="2" t="inlineStr">
+      <c r="F160" s="2" t="inlineStr">
         <is>
           <t>1. Look for the department-assigned Office staff member among the grid rows.
 2. Look for the staff member with no department.</t>
         </is>
       </c>
-      <c r="G161" s="2" t="inlineStr">
+      <c r="G160" s="2" t="inlineStr">
         <is>
           <t>1. The department-assigned staff member appears as a technician row - row presence is controlled by the department on the staff record, NOT by role permission.
 2. The staff member without a department does not appear as a row.</t>
         </is>
       </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md §14.4</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Clocking into work order line tasks is gated by the staff record's 'Time Clock' setting, not the permission model</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>1. Two staff members exist: one with the 'Time Clock' setting ON on their staff record, one with it OFF (set up; restore after).
+2. Both appear as schedule rows and have shifts on work order lines.</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr">
+        <is>
+          <t>1. As (or with) the Time-Clock-ON staff member, attempt to clock into their work order line task.
+2. As (or with) the Time-Clock-OFF staff member, attempt the same.</t>
+        </is>
+      </c>
+      <c r="G161" s="2" t="inlineStr">
+        <is>
+          <t>1. The Time-Clock-ON staff member can clock in.
+2. The Time-Clock-OFF staff member cannot - the ability is controlled by the staff-record setting, not by the Schedule permission tier.</t>
+        </is>
+      </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §14.4</t>
+          <t>requirements.md §14.4 (Time Clock setting)</t>
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr"/>
@@ -8360,7 +8358,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>Clocking into work order line tasks is gated by the staff record's 'Time Clock' setting, not the permission model</t>
+          <t>With Work Orders: View OFF, work-order-derived details on shifts (customer, lines, money fields) are hidden or masked</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -8370,173 +8368,126 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>1. Two staff members exist: one with the 'Time Clock' setting ON on their staff record, one with it OFF (set up; restore after).
-2. Both appear as schedule rows and have shifts on work order lines.</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>1. As (or with) the Time-Clock-ON staff member, attempt to clock into their work order line task.
-2. As (or with) the Time-Clock-OFF staff member, attempt the same.</t>
-        </is>
-      </c>
-      <c r="G162" s="2" t="inlineStr">
-        <is>
-          <t>1. The Time-Clock-ON staff member can clock in.
-2. The Time-Clock-OFF staff member cannot - the ability is controlled by the staff-record setting, not by the Schedule permission tier.</t>
-        </is>
-      </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.4 (Time Clock setting)</t>
-        </is>
-      </c>
-      <c r="I162" s="2" t="inlineStr"/>
-      <c r="J162" s="2" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
-        <is>
-          <t>With Work Orders: View OFF, work-order-derived details on shifts (customer, lines, money fields) are hidden or masked</t>
-        </is>
-      </c>
-      <c r="B163" s="2" t="inlineStr">
-        <is>
-          <t>Permissions</t>
-        </is>
-      </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="E163" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule access but Work Orders: View OFF (assign a suitable role; restore after).
 2. Shifts already exist on the grid, created by a fully-permissioned user, for units that have customers, scheduled lines, and a VIN.
 3. You are signed in AS that user on a desktop browser, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr">
+      <c r="F162" s="2" t="inlineStr">
         <is>
           <t>1. Look at a shift block on the grid and read its text lines.
 2. Hover the shift for its tooltip.
 3. Open the shift's detail modal and read the work-order-derived fields.</t>
         </is>
       </c>
-      <c r="G163" s="2" t="inlineStr">
+      <c r="G162" s="2" t="inlineStr">
         <is>
           <t>1. Work-order-derived details (customer, the scheduled line list, and any money-bearing fields) are hidden or masked wherever they would normally appear - on the block, in the tooltip, and in the modal.
 2. The schedule structure itself (the shift's day, time, and technician) stays visible so the grid remains usable.
 3. This extends the sidebar behavior (the work order list and drill-down are hidden) to the work-order data surfaced on the shifts themselves.</t>
         </is>
       </c>
-      <c r="H163" s="2" t="inlineStr">
+      <c r="H162" s="2" t="inlineStr">
         <is>
           <t>requirements.md §14.2 (Work Orders: View dependency)</t>
         </is>
       </c>
-      <c r="I163" s="2" t="inlineStr"/>
-      <c r="J163" s="2" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
+      <c r="I162" s="2" t="inlineStr"/>
+      <c r="J162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
         <is>
           <t>Planned hours across technicians may exceed the estimate - accepted without error</t>
         </is>
       </c>
-      <c r="B164" s="2" t="inlineStr">
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D164" s="2" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E164" s="2" t="inlineStr">
+      <c r="E163" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A work order line with a 40h estimate exists.</t>
         </is>
       </c>
-      <c r="F164" s="2" t="inlineStr">
+      <c r="F163" s="2" t="inlineStr">
         <is>
           <t>1. Spread the full estimate onto technician A.
 2. Spread the full estimate of the SAME work order onto technician B.
 3. Look for any warning or error about exceeding the estimate.</t>
         </is>
       </c>
-      <c r="G164" s="2" t="inlineStr">
+      <c r="G163" s="2" t="inlineStr">
         <is>
           <t>1. Both series are created - 80 planned hours against a 40h estimate is accepted.
 2. No error or blocking warning appears - this is expected behavior because progress is driven by clocked-in time, and scheduled hours, the estimate, and actual hours are three separate quantities that are not forced to reconcile.</t>
         </is>
       </c>
-      <c r="H164" s="2" t="inlineStr">
+      <c r="H163" s="2" t="inlineStr">
         <is>
           <t>requirements.md §12, §4.5</t>
         </is>
       </c>
-      <c r="I164" s="2" t="inlineStr"/>
-      <c r="J164" s="2" t="inlineStr"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="inlineStr">
+      <c r="I163" s="2" t="inlineStr"/>
+      <c r="J163" s="2" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>Below 960px the grid scrolls horizontally, and the sidebar collapses on narrow viewports</t>
         </is>
       </c>
-      <c r="B165" s="2" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D165" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E165" s="2" t="inlineStr">
+      <c r="E164" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
 2. You are on the Schedule page in week view with shifts visible.</t>
         </is>
       </c>
-      <c r="F165" s="2" t="inlineStr">
+      <c r="F164" s="2" t="inlineStr">
         <is>
           <t>1. Resize the browser window to just under 960px wide.
 2. Try to reach the right-hand days of the grid.
 3. Narrow the window further and watch the sidebar.</t>
         </is>
       </c>
-      <c r="G165" s="2" t="inlineStr">
+      <c r="G164" s="2" t="inlineStr">
         <is>
           <t>1. Below the 960px minimum supported width, the grid scrolls horizontally rather than breaking.
 2. All days remain reachable by horizontal scroll.
@@ -8544,210 +8495,210 @@
 4. No content becomes permanently unreachable and nothing errors.</t>
         </is>
       </c>
-      <c r="H165" s="2" t="inlineStr">
+      <c r="H164" s="2" t="inlineStr">
         <is>
           <t>requirements.md §11 (Responsiveness)</t>
         </is>
       </c>
-      <c r="I165" s="2" t="inlineStr"/>
-      <c r="J165" s="2" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
+      <c r="I164" s="2" t="inlineStr"/>
+      <c r="J164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
         <is>
           <t>The sidebar work order list and line drill-down stay smooth with 50+ items</t>
         </is>
       </c>
-      <c r="B166" s="2" t="inlineStr">
+      <c r="B165" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E166" s="2" t="inlineStr">
+      <c r="E165" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
 2. 50 or more open work orders exist (seed ZZAUTOTEST orders if the environment lacks them), including one order with many approved lines.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr">
+      <c r="F165" s="2" t="inlineStr">
         <is>
           <t>1. Scroll the full work order list top to bottom quickly.
 2. Open the many-line order's drill-down and scroll it.
 3. Type in the search while the long list is shown.</t>
         </is>
       </c>
-      <c r="G166" s="2" t="inlineStr">
+      <c r="G165" s="2" t="inlineStr">
         <is>
           <t>1. Scrolling stays smooth with no long freezes or blank stretches that fail to fill in (the list virtualizes at 50+ items).
 2. The drill-down behaves the same with many lines.
 3. Search stays responsive on the long list.</t>
         </is>
       </c>
-      <c r="H166" s="2" t="inlineStr">
+      <c r="H165" s="2" t="inlineStr">
         <is>
           <t>requirements.md §11 (Performance - virtualization)</t>
         </is>
       </c>
-      <c r="I166" s="2" t="inlineStr"/>
-      <c r="J166" s="2" t="inlineStr"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
+      <c r="I165" s="2" t="inlineStr"/>
+      <c r="J165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
         <is>
           <t>The grid renders smoothly at full load - 15 technicians × 7 days with several shifts per cell</t>
         </is>
       </c>
-      <c r="B167" s="2" t="inlineStr">
+      <c r="B166" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E167" s="2" t="inlineStr">
+      <c r="E166" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
 2. The schedule is loaded to roughly the spec's stated scale: around 15 technician rows across a week with several shifts per cell (seed ZZAUTOTEST shifts as needed).
 3. You are on the Schedule page in week view.</t>
         </is>
       </c>
-      <c r="F167" s="2" t="inlineStr">
+      <c r="F166" s="2" t="inlineStr">
         <is>
           <t>1. Scroll the grid vertically and horizontally.
 2. Switch between Day, Week, and Month.
 3. Hover several blocks and open/close a modal.</t>
         </is>
       </c>
-      <c r="G167" s="2" t="inlineStr">
+      <c r="G166" s="2" t="inlineStr">
         <is>
           <t>1. The grid renders and scrolls smoothly at this scale.
 2. View switches complete without long hangs.
 3. Tooltips and modals stay responsive.</t>
         </is>
       </c>
-      <c r="H167" s="2" t="inlineStr">
+      <c r="H166" s="2" t="inlineStr">
         <is>
           <t>requirements.md §11 (Performance)</t>
         </is>
       </c>
-      <c r="I167" s="2" t="inlineStr"/>
-      <c r="J167" s="2" t="inlineStr"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
+      <c r="I166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
         <is>
           <t>Shop closures block the spread step from placing shifts on those days</t>
         </is>
       </c>
-      <c r="B168" s="2" t="inlineStr">
+      <c r="B167" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E168" s="2" t="inlineStr">
+      <c r="E167" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shop closure (holiday/inventory day) is defined at the shop level on a working weekday inside the planned spread window (set it up; remove after).
 3. A large job (multi-day scope) is ready to spread.</t>
         </is>
       </c>
-      <c r="F168" s="2" t="inlineStr">
+      <c r="F167" s="2" t="inlineStr">
         <is>
           <t>1. Open the spread step across the window containing the closure.
 2. Expand the preview and find the closure day.
 3. Confirm the spread and check the grid.</t>
         </is>
       </c>
-      <c r="G168" s="2" t="inlineStr">
+      <c r="G167" s="2" t="inlineStr">
         <is>
           <t>1. The preview shows the closure day struck through with its reason.
 2. No shift is placed on the closure day - the series flows around it.
 3. The series' end date extends accordingly (the skipped day's hours land on later working days).</t>
         </is>
       </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>requirements.md §12 (Shop closures), §4.5</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr"/>
+      <c r="J167" s="2" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>Scheduled hours, the estimate, and actual (clocked) hours are three separate quantities that are not forced to reconcile</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>Edge Cases and Responsiveness</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in on a desktop browser with Schedule: Edit.
+2. A line has estimate 10h; a technician has 6h scheduled against it and some different amount of time actually clocked (seed what is possible).</t>
+        </is>
+      </c>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the shift's detail modal.
+2. Compare the scheduled hours, the estimate, and the logged/actual time.</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>1. All three quantities are shown/derivable and may differ from one another.
+2. Nothing forces them to match - no error, no auto-correction (progress is driven by clocked-in time).</t>
+        </is>
+      </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §12 (Shop closures), §4.5</t>
+          <t>requirements.md §4.5 (three separate quantities), §12</t>
         </is>
       </c>
       <c r="I168" s="2" t="inlineStr"/>
       <c r="J168" s="2" t="inlineStr"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>Scheduled hours, the estimate, and actual (clocked) hours are three separate quantities that are not forced to reconcile</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
-        <is>
-          <t>Edge Cases and Responsiveness</t>
-        </is>
-      </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>1. You are signed in on a desktop browser with Schedule: Edit.
-2. A line has estimate 10h; a technician has 6h scheduled against it and some different amount of time actually clocked (seed what is possible).</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the shift's detail modal.
-2. Compare the scheduled hours, the estimate, and the logged/actual time.</t>
-        </is>
-      </c>
-      <c r="G169" s="2" t="inlineStr">
-        <is>
-          <t>1. All three quantities are shown/derivable and may differ from one another.
-2. Nothing forces them to match - no error, no auto-correction (progress is driven by clocked-in time).</t>
-        </is>
-      </c>
-      <c r="H169" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §4.5 (three separate quantities), §12</t>
-        </is>
-      </c>
-      <c r="I169" s="2" t="inlineStr"/>
-      <c r="J169" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Schedule: author 10 new-scope cases (Working Hours x7, Week Export x2, New WO shortcut) + regen deliverables with Rule-20 refs (local)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/schedule-v1-testrail-import.xlsx
+++ b/testrail-import/schedule-v1-testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J168"/>
+  <dimension ref="A1:J178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -528,7 +528,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3</t>
+          <t>SV-8686 (§3)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -575,7 +575,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3, §3.1, §3.2</t>
+          <t>SV-8686 (§3, §3.1, §3.2)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.2, §6</t>
+          <t>SV-8686 (§3.2, §6)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -675,7 +675,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.2, §14.4</t>
+          <t>SV-8686 (§3.2, §14.4)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -723,7 +723,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.2</t>
+          <t>SV-8686 (§3.2)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -769,7 +769,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.2</t>
+          <t>SV-8686 (§3.2)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -818,7 +818,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.2, §4.2</t>
+          <t>SV-8686 (§3.2, §4.2)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -866,7 +866,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1, §5.2</t>
+          <t>SV-8687 (§3.1, §5.2)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.2</t>
+          <t>SV-8687 (§5.2)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -963,7 +963,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1, §5.2</t>
+          <t>SV-8687 (§3.1, §5.2)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -1012,7 +1012,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.2</t>
+          <t>SV-8687 (§5.2)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1, §5.1</t>
+          <t>SV-8687 (§3.1, §5.1)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Work order card anatomy)</t>
+          <t>SV-8687 (§3.1 (Work order card anatomy))</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Sidebar search)</t>
+          <t>SV-8687 (§3.1 (Sidebar search))</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Sidebar search, Work order card anatomy)</t>
+          <t>SV-8687 (§3.1 (Sidebar search, Work order card anatomy))</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Sidebar search)</t>
+          <t>SV-8687 (§3.1 (Sidebar search))</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (derived - search behavior with no matches)</t>
+          <t>SV-8687 (§3.1 (derived - search behavior with no matches))</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>The 'Filter' button opens Assignment / Status / Priority filter groups and shows an active-count badge</t>
+          <t>The 'Filters' button opens Assignment / Status / Priority filter groups</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1345,21 +1345,21 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>1. Click the 'Filter' button on the sidebar.
+          <t>1. Click the 'Filters' button on the sidebar.
 2. Read the filter groups offered.
-3. Apply one filter option and look at the 'Filter' button.</t>
+3. Apply one filter option and look at the 'Filters' button.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>1. The filter panel offers three groups: Assignment (Assigned, Unassigned), Status (the work order statuses supported in the app), and Priority (High, Medium, Low).
 2. Applying a filter narrows the flat card list.
-3. The 'Filter' button shows a badge with the number of active filters.</t>
+3. The 'Filters' button shows a badge with the number of active filters.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.1</t>
+          <t>SV-8687 (§5.1)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.1, §3.1</t>
+          <t>SV-8687 (§5.1, §3.1)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1459,7 +1459,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.1</t>
+          <t>SV-8687 (§5.1)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1508,7 +1508,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.1</t>
+          <t>SV-8687 (§5.1)</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.1</t>
+          <t>SV-8687 (§5.1)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §5.1</t>
+          <t>SV-8687 (§5.1)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Line drill-down)</t>
+          <t>SV-8687 (§3.1 (Line drill-down))</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Line drill-down)</t>
+          <t>SV-8687 (§3.1 (Line drill-down))</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Line drill-down - approved-only)</t>
+          <t>SV-8687 (§3.1 (Line drill-down - approved-only))</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Line drill-down), §8.1 (Line labor roster - no cap)</t>
+          <t>SV-8687 (§3.1 (Line drill-down), §8.1 (Line labor roster - no cap))</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Line drill-down - Needs techs badge)</t>
+          <t>SV-8687 (§3.1 (Line drill-down - Needs techs badge))</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1 (Line search)</t>
+          <t>SV-8687 (§3.1 (Line search))</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.1, §5.1 (drill-down filters)</t>
+          <t>SV-8687 (§3.1, §5.1 (drill-down filters))</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.1 (Single-line work order), §1.2 (roster sync), §7 (toast)</t>
+          <t>SV-8688 (§4.1 (Single-line work order), §1.2 (roster sync), §7 (toast))</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.1 (Multi-line work order), §4.3</t>
+          <t>SV-8688 (§4.1 (Multi-line work order), §4.3)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.1 (Specific line drag)</t>
+          <t>SV-8688 (§4.1 (Specific line drag))</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2148,7 +2148,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.1 (Large job), §4.5</t>
+          <t>SV-8688 (§4.1 (Large job), §4.5)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.1 (spread step is conditional)</t>
+          <t>SV-8688 (§4.1 (spread step is conditional))</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2245,7 +2245,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Drag feedback)</t>
+          <t>SV-8688 (§7 (Drag feedback))</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2294,7 +2294,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §1.2 (Goals - roster sync), §4.3 (roster add), §7</t>
+          <t>SV-8688 (§1.2 (Goals - roster sync), §4.3 (roster add), §7)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2342,7 +2342,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Keyboard support - click-to-arm), §11 (Accessibility)</t>
+          <t>SV-8688 (§7 (Keyboard support - click-to-arm), §11 (Accessibility))</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.3</t>
+          <t>SV-8689 (§4.3)</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.3, §4.4</t>
+          <t>SV-8689 (§4.3, §4.4)</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2490,7 +2490,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.3 (Individual line rows - fast path)</t>
+          <t>SV-8689 (§4.3 (Individual line rows - fast path))</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2538,7 +2538,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.3</t>
+          <t>SV-8689 (§4.3)</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2589,7 +2589,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.3 (Select multiple)</t>
+          <t>SV-8689 (§4.3 (Select multiple))</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.3 (Select all shortcut, Cancel)</t>
+          <t>SV-8689 (§4.3 (Select all shortcut, Cancel))</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2</t>
+          <t>SV-8688 (§4.2)</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2</t>
+          <t>SV-8688 (§4.2)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2</t>
+          <t>SV-8688 (§4.2)</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -2830,7 +2830,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2 (day view drop position)</t>
+          <t>SV-8688 (§4.2 (day view drop position))</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2 (Unassigned shifts), §3.2</t>
+          <t>SV-8688 (§4.2 (Unassigned shifts), §3.2)</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2</t>
+          <t>SV-8688 (§4.2)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §3.2 (Unassigned placeholder), §4.2</t>
+          <t>SV-8688 (§3.2 (Unassigned placeholder), §4.2)</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3025,7 +3025,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.2, §12</t>
+          <t>SV-8688 (§4.2, §12)</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3074,7 +3074,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5</t>
+          <t>SV-8691 (§4.5)</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -3121,7 +3121,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5</t>
+          <t>SV-8691 (§4.5)</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (How much to schedule)</t>
+          <t>SV-8691 (§4.5 (How much to schedule))</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (progressive disclosure)</t>
+          <t>SV-8691 (§4.5 (progressive disclosure))</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (progressive disclosure)</t>
+          <t>SV-8691 (§4.5 (progressive disclosure))</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (Start date)</t>
+          <t>SV-8691 (§4.5 (Start date))</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr"/>
@@ -3325,7 +3325,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Spread uses the technician's own working hours and skips weekends and shop closures - the end date is emergent</t>
+          <t>Spread uses the tech's working hours; skips weekends only when hours not set</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3360,13 +3360,14 @@
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>1. Daily shifts are sized to the technician's own working hours (8h each in the example).
-2. No shifts are placed on Saturday, Sunday, or the shop closure day.
-3. The end date is a result of the daily distribution (for 40h at 8h/day starting Monday with one closure, the series extends one extra working day).</t>
+2. Weekends are skipped ONLY when the technician has no business hours set for them; if the tech has hours on a weekend day (e.g. Saturday hours) that day is NOT skipped.
+3. Shop closures and public holidays are NOT skipped in V1 - shifts can be placed on those days.
+4. The end date is a result of the daily distribution (for 40h at 8h/day starting Monday, the series ends on the fifth working day).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5, §12 (shop closures)</t>
+          <t>SV-8691 (§4.5, §12 (shop closures))</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -3415,7 +3416,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (Preview)</t>
+          <t>SV-8691 (§4.5 (Preview))</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
@@ -3465,7 +3466,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (Confirming), §4.6, §8.2</t>
+          <t>SV-8691 (§4.5 (Confirming), §4.6, §8.2)</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -3514,7 +3515,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.5 (independent per-tech spread), §12</t>
+          <t>SV-8691 (§4.5 (independent per-tech spread), §12)</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr"/>
@@ -3565,7 +3566,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.6 (Month view)</t>
+          <t>SV-8692 (§4.6 (Month view))</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
@@ -3616,7 +3617,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.6 (Week view)</t>
+          <t>SV-8692 (§4.6 (Week view))</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
@@ -3664,7 +3665,7 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.6 (Day view)</t>
+          <t>SV-8692 (§4.6 (Day view))</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr"/>
@@ -3714,7 +3715,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.6, §8.2</t>
+          <t>SV-8692 (§4.6, §8.2)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
@@ -3763,7 +3764,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.4</t>
+          <t>SV-8690 (§4.4)</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
@@ -3813,7 +3814,7 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.4, §12</t>
+          <t>SV-8690 (§4.4, §12)</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr"/>
@@ -3863,7 +3864,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.4, §9 (VIN option)</t>
+          <t>SV-8690 (§4.4, §9 (VIN option))</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr"/>
@@ -3872,7 +3873,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Block color is tied to the work order - blocks from the same order share a color</t>
+          <t>Shift blocks default to blue; a custom colour can be set per shift</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -3899,20 +3900,21 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>1. Compare the colors of the two blocks from the same work order.
-2. Compare them with the other order's block.</t>
+          <t>1. Look at a newly created shift block's colour.
+2. Open the shift detail modal and set a custom colour via the colour picker.
+3. Compare that shift with another shift from the same work order.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>1. The two blocks from the same work order share the same color.
-2. Blocks from different work orders can have different colors.
-3. By default blocks are blue (the default shift color) unless a custom color was chosen.</t>
+          <t>1. By default every shift block is blue (the default shift colour).
+2. A custom colour can be assigned per shift via the colour picker in the detail modal.
+3. Colour is per shift - it is NOT tied to the work order, so two shifts from the same order do not automatically share a colour.</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.4, §10</t>
+          <t>SV-8690 (§4.4, §10)</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr"/>
@@ -3961,7 +3963,7 @@
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.4</t>
+          <t>SV-8690 (§4.4)</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr"/>
@@ -4009,7 +4011,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.7</t>
+          <t>SV-8693 (§4.7)</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr"/>
@@ -4057,7 +4059,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.7, §4.11</t>
+          <t>SV-8693 (§4.7, §4.11)</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr"/>
@@ -4107,7 +4109,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.7</t>
+          <t>SV-8693 (§4.7)</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr"/>
@@ -4157,7 +4159,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.7</t>
+          <t>SV-8693 (§4.7)</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr"/>
@@ -4205,7 +4207,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §12 (edge case), §4.7</t>
+          <t>SV-8693 (§12 (edge case), §4.7)</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr"/>
@@ -4254,7 +4256,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8 (Auto-scroll to business hours)</t>
+          <t>SV-8694 (§4.8 (Auto-scroll to business hours))</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr"/>
@@ -4303,7 +4305,7 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8</t>
+          <t>SV-8694 (§4.8)</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr"/>
@@ -4352,7 +4354,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8 (Sticky header bar)</t>
+          <t>SV-8694 (§4.8 (Sticky header bar))</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr"/>
@@ -4403,7 +4405,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8 (Horizontal drag), §7 (toast)</t>
+          <t>SV-8694 (§4.8 (Horizontal drag), §7 (toast))</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
@@ -4454,7 +4456,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8 (Edge resize)</t>
+          <t>SV-8694 (§4.8 (Edge resize))</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr"/>
@@ -4503,7 +4505,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8 (Now line)</t>
+          <t>SV-8694 (§4.8 (Now line))</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr"/>
@@ -4552,7 +4554,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.8 (Lane height with VIN)</t>
+          <t>SV-8694 (§4.8 (Lane height with VIN))</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr"/>
@@ -4601,7 +4603,7 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9, §9 (VIN always in modal)</t>
+          <t>SV-8695 (§4.9, §9 (VIN always in modal))</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr"/>
@@ -4652,7 +4654,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9</t>
+          <t>SV-8695 (§4.9)</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -4701,7 +4703,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9</t>
+          <t>SV-8695 (§4.9)</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr"/>
@@ -4751,7 +4753,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9, §4.4</t>
+          <t>SV-8695 (§4.9, §4.4)</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -4800,7 +4802,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9 (Estimated hours with inline edit)</t>
+          <t>SV-8695 (§4.9 (Estimated hours with inline edit))</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -4850,7 +4852,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9 (Notes: add, edit, and delete per work order)</t>
+          <t>SV-8695 (§4.9 (Notes: add, edit, and delete per work order))</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr"/>
@@ -4901,7 +4903,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9 (conflict banner + Adjust)</t>
+          <t>SV-8695 (§4.9 (conflict banner + Adjust))</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
@@ -4950,7 +4952,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.9 (Actions), §7</t>
+          <t>SV-8695 (§4.9 (Actions), §7)</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -4959,7 +4961,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Create an event via right-click 'New Event' on a grid cell</t>
+          <t>Create an event via right-click 'Create Event' on a grid cell</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -4986,13 +4988,13 @@
       <c r="F93" s="2" t="inlineStr">
         <is>
           <t>1. Right-click a technician's cell on a working day.
-2. Choose 'New Event' from the context menu.
+2. Choose 'Create Event' from the context menu.
 3. Fill in a name (for example 'ZZAUTOTEST stand-up'), keep the date/times offered, and save.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>1. The right-click context menu contains 'New Event'.
+          <t>1. The right-click context menu contains 'Create Event'.
 2. The event modal opens with the clicked cell's technician and date pre-set.
 3. Saving creates an event block on that technician's day.
 4. A toast with Undo appears.</t>
@@ -5000,7 +5002,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10, §7 (right-click menu)</t>
+          <t>SV-8696 (§4.10, §7 (right-click menu))</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
@@ -5049,7 +5051,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10 (day-view click-to-create, live preview)</t>
+          <t>SV-8696 (§4.10 (day-view click-to-create, live preview))</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
@@ -5098,7 +5100,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10 (Event modal)</t>
+          <t>SV-8696 (§4.10 (Event modal))</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -5146,7 +5148,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10, §8.1 (Event allDay field)</t>
+          <t>SV-8696 (§4.10, §8.1 (Event allDay field))</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
@@ -5196,7 +5198,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10 (Drag-and-drop to reassign/move), §7 (toast)</t>
+          <t>SV-8696 (§4.10 (Drag-and-drop to reassign/move), §7 (toast))</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -5244,7 +5246,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10 (Event card anatomy)</t>
+          <t>SV-8696 (§4.10 (Event card anatomy))</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
@@ -5294,7 +5296,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10 (Event color), §10</t>
+          <t>SV-8696 (§4.10 (Event color), §10)</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
@@ -5344,7 +5346,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.10 (Events), §4.11, §4.12</t>
+          <t>SV-8696 (§4.10 (Events), §4.11, §4.12)</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
@@ -5395,7 +5397,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11 (Double-booked)</t>
+          <t>SV-8697 (§4.11 (Double-booked))</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
@@ -5444,7 +5446,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11 (Weekend shift)</t>
+          <t>SV-8697 (§4.11 (Weekend shift))</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
@@ -5493,7 +5495,7 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11 (Before hours)</t>
+          <t>SV-8697 (§4.11 (Before hours))</t>
         </is>
       </c>
       <c r="I103" s="2" t="inlineStr"/>
@@ -5542,7 +5544,7 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11 (After hours)</t>
+          <t>SV-8697 (§4.11 (After hours))</t>
         </is>
       </c>
       <c r="I104" s="2" t="inlineStr"/>
@@ -5593,7 +5595,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11, §6 (Conflict pill)</t>
+          <t>SV-8697 (§4.11, §6 (Conflict pill))</t>
         </is>
       </c>
       <c r="I105" s="2" t="inlineStr"/>
@@ -5641,7 +5643,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11 (Clicking a conflict navigates)</t>
+          <t>SV-8697 (§4.11 (Clicking a conflict navigates))</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr"/>
@@ -5689,7 +5691,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.11 (styling rule), §4.12</t>
+          <t>SV-8697 (§4.11 (styling rule), §4.12)</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr"/>
@@ -5740,7 +5742,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.12 (Blue fill)</t>
+          <t>SV-8698 (§4.12 (Blue fill))</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr"/>
@@ -5787,7 +5789,7 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.12 (Amber spill)</t>
+          <t>SV-8698 (§4.12 (Amber spill))</t>
         </is>
       </c>
       <c r="I109" s="2" t="inlineStr"/>
@@ -5835,7 +5837,7 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.12 (OT tag), §11 (not color-only)</t>
+          <t>SV-8698 (§4.12 (OT tag), §11 (not color-only))</t>
         </is>
       </c>
       <c r="I110" s="2" t="inlineStr"/>
@@ -5884,7 +5886,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.12 (Hover tooltip)</t>
+          <t>SV-8698 (§4.12 (Hover tooltip))</t>
         </is>
       </c>
       <c r="I111" s="2" t="inlineStr"/>
@@ -5933,7 +5935,7 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.13 (Shift tooltip)</t>
+          <t>SV-8695 (§4.13 (Shift tooltip))</t>
         </is>
       </c>
       <c r="I112" s="2" t="inlineStr"/>
@@ -5980,7 +5982,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.13 (Shift tooltip - conflict)</t>
+          <t>SV-8695 (§4.13 (Shift tooltip - conflict))</t>
         </is>
       </c>
       <c r="I113" s="2" t="inlineStr"/>
@@ -6028,7 +6030,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.13 (Event tooltip)</t>
+          <t>SV-8695 (§4.13 (Event tooltip))</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr"/>
@@ -6080,7 +6082,7 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.13 (Behavior)</t>
+          <t>SV-8695 (§4.13 (Behavior))</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr"/>
@@ -6129,7 +6131,7 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §4.13 (flip/shift to stay in viewport)</t>
+          <t>SV-8695 (§4.13 (flip/shift to stay in viewport))</t>
         </is>
       </c>
       <c r="I116" s="2" t="inlineStr"/>
@@ -6176,7 +6178,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §6 (Today button)</t>
+          <t>SV-8686 (§6 (Today button))</t>
         </is>
       </c>
       <c r="I117" s="2" t="inlineStr"/>
@@ -6226,7 +6228,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §6 (Left/right arrows, Date label)</t>
+          <t>SV-8686 (§6 (Left/right arrows, Date label))</t>
         </is>
       </c>
       <c r="I118" s="2" t="inlineStr"/>
@@ -6277,7 +6279,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §6 (Search)</t>
+          <t>SV-8686 (§6 (Search))</t>
         </is>
       </c>
       <c r="I119" s="2" t="inlineStr"/>
@@ -6286,7 +6288,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>'Filter and Display' is a checkbox-style dropdown combining department toggles, My Shifts, and VIN</t>
+          <t>'Filter &amp; Display' dropdown combines department toggles, My Shifts, and VIN</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -6312,7 +6314,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>1. Open the 'Filter and Display' dropdown in the grid toolbar.
+          <t>1. Open the 'Filter &amp; Display' dropdown in the grid toolbar.
 2. Read its contents and default states.</t>
         </is>
       </c>
@@ -6325,7 +6327,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §6, §9 (Filter and Display dropdown)</t>
+          <t>SV-8700 (§6, §9 (Filter and Display dropdown))</t>
         </is>
       </c>
       <c r="I120" s="2" t="inlineStr"/>
@@ -6375,7 +6377,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (Department toggles)</t>
+          <t>SV-8700 (§9 (Department toggles))</t>
         </is>
       </c>
       <c r="I121" s="2" t="inlineStr"/>
@@ -6425,7 +6427,7 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (My Shifts), §14.3</t>
+          <t>SV-8700 (§9 (My Shifts), §14.3)</t>
         </is>
       </c>
       <c r="I122" s="2" t="inlineStr"/>
@@ -6475,7 +6477,7 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (VIN), §4.4</t>
+          <t>SV-8700 (§9 (VIN), §4.4)</t>
         </is>
       </c>
       <c r="I123" s="2" t="inlineStr"/>
@@ -6522,7 +6524,7 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §6, §9 (View Options popover)</t>
+          <t>SV-8700 (§6, §9 (View Options popover))</t>
         </is>
       </c>
       <c r="I124" s="2" t="inlineStr"/>
@@ -6572,7 +6574,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (Business Hours), §4.8 (Business-hours shading)</t>
+          <t>SV-8700 (§9 (Business Hours), §4.8 (Business-hours shading))</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr"/>
@@ -6621,7 +6623,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (Capacity Bars), §4.12</t>
+          <t>SV-8700 (§9 (Capacity Bars), §4.12)</t>
         </is>
       </c>
       <c r="I126" s="2" t="inlineStr"/>
@@ -6670,7 +6672,7 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (Events)</t>
+          <t>SV-8700 (§9 (Events))</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr"/>
@@ -6719,7 +6721,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (Tech Hours)</t>
+          <t>SV-8700 (§9 (Tech Hours))</t>
         </is>
       </c>
       <c r="I128" s="2" t="inlineStr"/>
@@ -6768,7 +6770,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §9 (Saturday, Sunday), §3.2 (Week view)</t>
+          <t>SV-8700 (§9 (Saturday, Sunday), §3.2 (Week view))</t>
         </is>
       </c>
       <c r="I129" s="2" t="inlineStr"/>
@@ -6819,7 +6821,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Shift reassignment), §12</t>
+          <t>SV-8695 (§7 (Shift reassignment), §12)</t>
         </is>
       </c>
       <c r="I130" s="2" t="inlineStr"/>
@@ -6828,7 +6830,7 @@
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>Right-click on any grid cell opens a context menu with New Shift, New Event, and View Day</t>
+          <t>Right-click a grid cell opens a menu with Create Event and New Work Order</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -6861,13 +6863,13 @@
       <c r="G131" s="2" t="inlineStr">
         <is>
           <t>1. A context menu opens at the cell.
-2. It contains: 'New Shift', 'New Event', and 'View Day'.
+2. It contains: 'Create Event' and 'New Work Order'.
 3. The browser's own right-click menu does not appear instead.</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Right-click context menu)</t>
+          <t>SV-8700 (§7 (Right-click context menu))</t>
         </is>
       </c>
       <c r="I131" s="2" t="inlineStr"/>
@@ -6876,7 +6878,7 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>'View Day' in the context menu opens day view for that cell's date</t>
+          <t>'View Day' is no longer offered in the grid cell context menu</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6902,19 +6904,19 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>1. Right-click a cell on a specific day.
-2. Choose 'View Day'.</t>
+          <t>1. Right-click a technician's grid cell.
+2. Read the menu items.</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>1. The grid switches to day view showing that cell's date.
-2. The toolbar date label and the Day/Week/Month control reflect the switch.</t>
+          <t>1. The context menu shows only 'Create Event' and 'New Work Order'.
+2. There is no 'View Day' item - it was removed from the menu.</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Right-click context menu - View Day)</t>
+          <t>SV-8700 (§7 (Right-click context menu - View Day))</t>
         </is>
       </c>
       <c r="I132" s="2" t="inlineStr"/>
@@ -6923,7 +6925,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>'New Shift' in the context menu starts shift creation for that technician and day</t>
+          <t>'New Shift' is no longer offered in the grid cell context menu</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -6950,19 +6952,19 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>1. Right-click a technician's cell and choose 'New Shift'.
-2. Complete the creation flow that opens.</t>
+          <t>1. Right-click a technician's grid cell.
+2. Read the menu items.</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>1. A shift-creation flow opens targeted at that technician and day.
-2. Completing it creates a shift in that cell, following the same scope/spread rules as drag-and-drop.</t>
+          <t>1. The context menu shows only 'Create Event' and 'New Work Order'.
+2. There is no 'New Shift' item - it was removed from the menu.</t>
         </is>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>requirements.md §7 (Right-click context menu - New Shift), §14.1 (creation via context menu)</t>
+          <t>SV-8700 (§7 (Right-click context menu - New Shift), §14.1 (creation via context menu))</t>
         </is>
       </c>
       <c r="I133" s="2" t="inlineStr"/>
@@ -6971,88 +6973,136 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
+          <t>'New Work Order' in the cell menu points the user to the Work Orders tab</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Reassignment and Context Menu</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>1. You are on the Schedule grid.
+2. The cell context menu shows 'Create Event' and 'New Work Order' ().</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>1. Right-click an empty grid cell.
+2. Choose 'New Work Order' from the menu.</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>1. The menu offers a 'New Work Order' item.
+2. Choosing it directs the user to create a work order (a toast / prompt pointing to the Work Orders tab).
+3. The exact target flow (toast or navigation) is confirmed during live testing.</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§7 / §4.10 New Work Order cell-menu shortcut)</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr"/>
+      <c r="J134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
           <t>Deleting a middle shift of a series asks for scope with all three options, each stating the hours returned</t>
         </is>
       </c>
-      <c r="B134" s="2" t="inlineStr">
+      <c r="B135" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C134" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D134" s="2" t="inlineStr">
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E134" s="2" t="inlineStr">
+      <c r="E135" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 3 shifts exists for one technician.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F134" s="2" t="inlineStr">
+      <c r="F135" s="2" t="inlineStr">
         <is>
           <t>1. Delete a MIDDLE shift of the series (via the detail modal's Delete).
 2. Read the scope options offered (do not confirm yet).</t>
         </is>
       </c>
-      <c r="G134" s="2" t="inlineStr">
+      <c r="G135" s="2" t="inlineStr">
         <is>
           <t>1. A scope prompt appears with three options: this shift only, this and everything after, and the whole series.
 2. Each option states its consequence in hours returned (spec's example format: 'returns 8h' / 'returns 56h').
 3. The prompt uses routine, lightweight styling - not alarming destructive styling.</t>
         </is>
       </c>
-      <c r="H134" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Series-aware deletion)</t>
-        </is>
-      </c>
-      <c r="I134" s="2" t="inlineStr"/>
-      <c r="J134" s="2" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="inlineStr">
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>SV-8692 (§7 (Series-aware deletion))</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr"/>
+      <c r="J135" s="2" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
         <is>
           <t>'This shift only' removes that day, the series keeps the gap, and the hours return to the estimate's remaining</t>
         </is>
       </c>
-      <c r="B135" s="2" t="inlineStr">
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C135" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D135" s="2" t="inlineStr">
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E135" s="2" t="inlineStr">
+      <c r="E136" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 3 shifts exists; note the total scheduled hours.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F135" s="2" t="inlineStr">
+      <c r="F136" s="2" t="inlineStr">
         <is>
           <t>1. Delete a middle shift with the 'this shift only' scope.
 2. Look at the series on the grid.
 3. Check the scheduled hours.</t>
         </is>
       </c>
-      <c r="G135" s="2" t="inlineStr">
+      <c r="G136" s="2" t="inlineStr">
         <is>
           <t>1. Only that day's shift is removed.
 2. The series keeps the gap - the remaining shifts do NOT shuffle to close it.
@@ -7060,148 +7110,148 @@
 4. An undo toast appears.</t>
         </is>
       </c>
-      <c r="H135" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (This shift only)</t>
-        </is>
-      </c>
-      <c r="I135" s="2" t="inlineStr"/>
-      <c r="J135" s="2" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="inlineStr">
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>SV-8692 (§7 (This shift only))</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
         <is>
           <t>'This and everything after' removes from the clicked shift onward, keeping earlier shifts</t>
         </is>
       </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B137" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E136" s="2" t="inlineStr">
+      <c r="E137" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 4 shifts exists.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F136" s="2" t="inlineStr">
+      <c r="F137" s="2" t="inlineStr">
         <is>
           <t>1. Delete the series' THIRD shift with the 'this and everything after' scope.
 2. Look at the series on the grid.</t>
         </is>
       </c>
-      <c r="G136" s="2" t="inlineStr">
+      <c r="G137" s="2" t="inlineStr">
         <is>
           <t>1. The third shift and every later shift of the series are removed.
 2. The first two shifts remain untouched.
 3. An undo toast appears.</t>
         </is>
       </c>
-      <c r="H136" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (This and everything after)</t>
-        </is>
-      </c>
-      <c r="I136" s="2" t="inlineStr"/>
-      <c r="J136" s="2" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="inlineStr">
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>SV-8692 (§7 (This and everything after))</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr"/>
+      <c r="J137" s="2" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
         <is>
           <t>'The whole series' removes all of the series' shifts for that technician</t>
         </is>
       </c>
-      <c r="B137" s="2" t="inlineStr">
+      <c r="B138" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C137" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D137" s="2" t="inlineStr">
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E137" s="2" t="inlineStr">
+      <c r="E138" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. The SAME work order has a series on technician A and an independent series on technician B.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F137" s="2" t="inlineStr">
+      <c r="F138" s="2" t="inlineStr">
         <is>
           <t>1. Delete one of technician A's series shifts with the 'whole series' scope.
 2. Look at both technicians' rows.</t>
         </is>
       </c>
-      <c r="G137" s="2" t="inlineStr">
+      <c r="G138" s="2" t="inlineStr">
         <is>
           <t>1. All of technician A's series shifts are removed.
 2. Technician B's independent series is untouched (the scope is per technician's series).
 3. An undo toast appears.</t>
         </is>
       </c>
-      <c r="H137" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (The whole series - 'for that technician')</t>
-        </is>
-      </c>
-      <c r="I137" s="2" t="inlineStr"/>
-      <c r="J137" s="2" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>SV-8692 (§7 (The whole series - 'for that technician'))</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr"/>
+      <c r="J138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
         <is>
           <t>Scope options adapt to position: first and last shifts of a series each show only two options</t>
         </is>
       </c>
-      <c r="B138" s="2" t="inlineStr">
+      <c r="B139" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E138" s="2" t="inlineStr">
+      <c r="E139" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A series of at least 3 shifts exists.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F138" s="2" t="inlineStr">
+      <c r="F139" s="2" t="inlineStr">
         <is>
           <t>1. Start deleting the FIRST shift of the series; read the options, then cancel.
 2. Start deleting the LAST shift; read the options, then cancel.
 3. Start deleting a MIDDLE shift; read the options, then cancel.</t>
         </is>
       </c>
-      <c r="G138" s="2" t="inlineStr">
+      <c r="G139" s="2" t="inlineStr">
         <is>
           <t>1. First shift: two options ('this and after' would equal 'whole series', so only two are shown).
 2. Last shift: two options ('this and after' would equal 'this only').
@@ -7209,91 +7259,91 @@
 4. Cancelling leaves the series unchanged in every case.</t>
         </is>
       </c>
-      <c r="H138" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (options adapt to position)</t>
-        </is>
-      </c>
-      <c r="I138" s="2" t="inlineStr"/>
-      <c r="J138" s="2" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="inlineStr">
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>SV-8692 (§7 (options adapt to position))</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr"/>
+      <c r="J139" s="2" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
         <is>
           <t>Deleting a standalone (non-series) shift does not ask for a series scope</t>
         </is>
       </c>
-      <c r="B139" s="2" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C139" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D139" s="2" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E139" s="2" t="inlineStr">
+      <c r="E140" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A single standalone shift (not part of any series) exists.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr">
+      <c r="F140" s="2" t="inlineStr">
         <is>
           <t>1. Delete the standalone shift.
 2. Watch what is asked.</t>
         </is>
       </c>
-      <c r="G139" s="2" t="inlineStr">
+      <c r="G140" s="2" t="inlineStr">
         <is>
           <t>1. No series-scope prompt appears (the scope question is only for shifts that belong to a series).
 2. The shift is deleted and an undo toast appears.</t>
         </is>
       </c>
-      <c r="H139" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (derived - scope prompt is for series shifts)</t>
-        </is>
-      </c>
-      <c r="I139" s="2" t="inlineStr"/>
-      <c r="J139" s="2" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="inlineStr">
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>SV-8692 (§7 (derived - scope prompt is for series shifts))</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
         <is>
           <t>Every create, delete, move, and reassign action produces a toast with an Undo option</t>
         </is>
       </c>
-      <c r="B140" s="2" t="inlineStr">
+      <c r="B141" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E140" s="2" t="inlineStr">
+      <c r="E141" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. Schedulable lines and an existing shift are available.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr">
+      <c r="F141" s="2" t="inlineStr">
         <is>
           <t>1. Create a shift - watch for a toast.
 2. Move a shift to another day - watch for a toast.
@@ -7301,98 +7351,98 @@
 4. Delete a shift - watch for a toast.</t>
         </is>
       </c>
-      <c r="G140" s="2" t="inlineStr">
+      <c r="G141" s="2" t="inlineStr">
         <is>
           <t>1. Each of the four actions produces a toast notification.
 2. Every toast offers an Undo option.</t>
         </is>
       </c>
-      <c r="H140" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Toast notifications), §11 (Undo)</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="inlineStr"/>
-      <c r="J140" s="2" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>The toast persists 4 to 7 seconds, stays while the cursor is over it, and dismisses on mouse-leave</t>
-        </is>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>SV-8688 (§7 (Toast notifications), §11 (Undo))</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr"/>
+      <c r="J141" s="2" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Toast lasts ~7s with Undo (about 4s without); stays on hover, goes on leave</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C141" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E141" s="2" t="inlineStr">
+      <c r="E142" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F141" s="2" t="inlineStr">
+      <c r="F142" s="2" t="inlineStr">
         <is>
           <t>1. Perform an action that shows a toast (for example move a shift) and let the toast sit untouched - time how long it stays.
 2. Trigger another toast and hold the cursor OVER it well past its normal lifetime.
 3. Move the cursor off the toast.</t>
         </is>
       </c>
-      <c r="G141" s="2" t="inlineStr">
-        <is>
-          <t>1. Untouched, the toast persists for roughly 4 to 7 seconds before dismissing.
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>1. Untouched, a toast that has an Undo action persists about 7 seconds; a toast without Undo persists about 4 seconds, before dismissing.
 2. While the cursor is over it, the toast stays (does not auto-dismiss).
 3. After the cursor leaves, it dismisses.</t>
         </is>
       </c>
-      <c r="H141" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Toast notifications), §11 (Undo)</t>
-        </is>
-      </c>
-      <c r="I141" s="2" t="inlineStr"/>
-      <c r="J141" s="2" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="inlineStr">
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>SV-8688 (§7 (Toast notifications), §11 (Undo))</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
         <is>
           <t>Undo restores the state before the action - for delete, move, and reassign</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="B143" s="2" t="inlineStr">
         <is>
           <t>Deletion, Series Scopes and Undo</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D142" s="2" t="inlineStr">
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E142" s="2" t="inlineStr">
+      <c r="E143" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. A shift exists; note its technician, day, and time.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
+      <c r="F143" s="2" t="inlineStr">
         <is>
           <t>1. Delete the shift, then click Undo on the toast.
 2. Move the shift to another day, then click Undo.
@@ -7400,7 +7450,7 @@
 4. Check the line's roster after the reassign undo.</t>
         </is>
       </c>
-      <c r="G142" s="2" t="inlineStr">
+      <c r="G143" s="2" t="inlineStr">
         <is>
           <t>1. Undo after delete: the shift is back exactly where it was.
 2. Undo after move: the shift returns to its original day/time.
@@ -7408,91 +7458,91 @@
 4. Every destructive action is undoable within the toast's lifetime.</t>
         </is>
       </c>
-      <c r="H142" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §11 (Undo), §7</t>
-        </is>
-      </c>
-      <c r="I142" s="2" t="inlineStr"/>
-      <c r="J142" s="2" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="2" t="inlineStr">
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>SV-8688 (§11 (Undo), §7)</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr"/>
+      <c r="J143" s="2" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
         <is>
           <t>Escape closes the topmost open modal or popover, following the stacking order</t>
         </is>
       </c>
-      <c r="B143" s="2" t="inlineStr">
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D143" s="2" t="inlineStr">
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E143" s="2" t="inlineStr">
+      <c r="E144" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr">
+      <c r="F144" s="2" t="inlineStr">
         <is>
           <t>1. Open the shift detail modal, then open a popover on top of it (for example the color picker or a filter/search popover elsewhere).
 2. Press Escape once.
 3. Press Escape again.</t>
         </is>
       </c>
-      <c r="G143" s="2" t="inlineStr">
+      <c r="G144" s="2" t="inlineStr">
         <is>
           <t>1. The FIRST Escape closes only the topmost layer (the popover), leaving the layer beneath open.
 2. The SECOND Escape closes the next layer down.
 3. Escape works anywhere on the schedule page as a global shortcut, following the defined stacking order (delete scope, reassign, spread, capacity, event modal, event view, line picker, shift detail, cell menu, calendar picker, customize, filters, search).</t>
         </is>
       </c>
-      <c r="H143" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Keyboard support - Escape)</t>
-        </is>
-      </c>
-      <c r="I143" s="2" t="inlineStr"/>
-      <c r="J143" s="2" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="inlineStr">
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§7 (Keyboard support - Escape))</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
         <is>
           <t>Within the shift modal, Escape first dismisses an open sub-picker before closing the modal itself</t>
         </is>
       </c>
-      <c r="B144" s="2" t="inlineStr">
+      <c r="B145" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C144" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D144" s="2" t="inlineStr">
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E144" s="2" t="inlineStr">
+      <c r="E145" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's detail modal is open.</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr">
+      <c r="F145" s="2" t="inlineStr">
         <is>
           <t>1. Open the color picker inside the modal, press Escape, and watch.
 2. Open the time picker, press Escape.
@@ -7500,50 +7550,50 @@
 4. With nothing open inside the modal, press Escape.</t>
         </is>
       </c>
-      <c r="G144" s="2" t="inlineStr">
+      <c r="G145" s="2" t="inlineStr">
         <is>
           <t>1. Escape with the color picker open closes only the color picker - the modal stays open.
 2. Same for the time picker and the note edit.
 3. Escape with no open sub-picker closes the modal itself.</t>
         </is>
       </c>
-      <c r="H144" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Escape within the shift modal)</t>
-        </is>
-      </c>
-      <c r="I144" s="2" t="inlineStr"/>
-      <c r="J144" s="2" t="inlineStr"/>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="inlineStr">
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§7 (Escape within the shift modal))</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr"/>
+      <c r="J145" s="2" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
         <is>
           <t>Enter confirms the active confirmable dialog (delete scope, reassign, spread, event create/edit)</t>
         </is>
       </c>
-      <c r="B145" s="2" t="inlineStr">
+      <c r="B146" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C145" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D145" s="2" t="inlineStr">
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E145" s="2" t="inlineStr">
+      <c r="E146" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Delete.
 2. Shifts/series and events exist to exercise the dialogs.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F145" s="2" t="inlineStr">
+      <c r="F146" s="2" t="inlineStr">
         <is>
           <t>1. Open the spread step for a large job, press Enter.
 2. Open the reassign dialog for a shift, choose a technician, press Enter.
@@ -7551,241 +7601,241 @@
 4. Open a series delete-scope prompt, select a scope, press Enter.</t>
         </is>
       </c>
-      <c r="G145" s="2" t="inlineStr">
+      <c r="G146" s="2" t="inlineStr">
         <is>
           <t>1. In each confirmable dialog, Enter confirms it - equivalent to clicking its confirm action.
 2. The confirmed action takes effect (spread created / reassigned / event saved / delete applied).</t>
         </is>
       </c>
-      <c r="H145" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Keyboard support - Enter)</t>
-        </is>
-      </c>
-      <c r="I145" s="2" t="inlineStr"/>
-      <c r="J145" s="2" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="2" t="inlineStr">
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§7 (Keyboard support - Enter))</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
         <is>
           <t>Enter does not fire inside textareas - multiline note editing works normally</t>
         </is>
       </c>
-      <c r="B146" s="2" t="inlineStr">
+      <c r="B147" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C146" s="2" t="inlineStr">
+      <c r="C147" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D146" s="2" t="inlineStr">
+      <c r="D147" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E146" s="2" t="inlineStr">
+      <c r="E147" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's detail modal is open with the note editor active.</t>
         </is>
       </c>
-      <c r="F146" s="2" t="inlineStr">
+      <c r="F147" s="2" t="inlineStr">
         <is>
           <t>1. Type a line of note text and press Enter.
 2. Type a second line.</t>
         </is>
       </c>
-      <c r="G146" s="2" t="inlineStr">
+      <c r="G147" s="2" t="inlineStr">
         <is>
           <t>1. Enter inserts a new line in the note - it does NOT confirm/close the dialog.
 2. The multiline note can be completed and saved normally.</t>
         </is>
       </c>
-      <c r="H146" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §7 (Enter does not fire inside textareas)</t>
-        </is>
-      </c>
-      <c r="I146" s="2" t="inlineStr"/>
-      <c r="J146" s="2" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="2" t="inlineStr">
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§7 (Enter does not fire inside textareas))</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr"/>
+      <c r="J147" s="2" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
         <is>
           <t>Modals trap focus and all interactive elements are keyboard-reachable</t>
         </is>
       </c>
-      <c r="B147" s="2" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>Keyboard Interactions</t>
         </is>
       </c>
-      <c r="C147" s="2" t="inlineStr">
+      <c r="C148" s="2" t="inlineStr">
         <is>
           <t>Accessibility</t>
         </is>
       </c>
-      <c r="D147" s="2" t="inlineStr">
+      <c r="D148" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E147" s="2" t="inlineStr">
+      <c r="E148" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's detail modal is open.</t>
         </is>
       </c>
-      <c r="F147" s="2" t="inlineStr">
+      <c r="F148" s="2" t="inlineStr">
         <is>
           <t>1. Press Tab repeatedly and watch where focus goes.
 2. Continue tabbing past the last control in the modal.
 3. Close the modal and Tab through the schedule page's toolbar and sidebar controls.</t>
         </is>
       </c>
-      <c r="G147" s="2" t="inlineStr">
+      <c r="G148" s="2" t="inlineStr">
         <is>
           <t>1. Focus moves through the modal's interactive elements with visible focus rings.
 2. Focus stays trapped inside the modal (wraps back to its first control) until the modal closes.
 3. On the page, toolbar and sidebar controls are reachable by keyboard.</t>
         </is>
       </c>
-      <c r="H147" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §11 (Accessibility)</t>
-        </is>
-      </c>
-      <c r="I147" s="2" t="inlineStr"/>
-      <c r="J147" s="2" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="2" t="inlineStr">
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§11 (Accessibility))</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
         <is>
           <t>Blue is the default color for all shifts, including long and multi-week jobs</t>
         </is>
       </c>
-      <c r="B148" s="2" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>Color System</t>
         </is>
       </c>
-      <c r="C148" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D148" s="2" t="inlineStr">
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E148" s="2" t="inlineStr">
+      <c r="E149" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F148" s="2" t="inlineStr">
+      <c r="F149" s="2" t="inlineStr">
         <is>
           <t>1. Create a normal single-day shift without touching any color option.
 2. Create a multi-week series without touching any color option.
 3. Look at both on the grid.</t>
         </is>
       </c>
-      <c r="G148" s="2" t="inlineStr">
+      <c r="G149" s="2" t="inlineStr">
         <is>
           <t>1. Both the single shift and the multi-week series render in the default blue.
 2. No special color is auto-applied to long jobs - blue is the default for ALL shifts.</t>
         </is>
       </c>
-      <c r="H148" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §10</t>
-        </is>
-      </c>
-      <c r="I148" s="2" t="inlineStr"/>
-      <c r="J148" s="2" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§10)</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr"/>
+      <c r="J149" s="2" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
         <is>
           <t>Choosing a color from the shift modal's picker recolors the shift with matching background, text, and accent tones</t>
         </is>
       </c>
-      <c r="B149" s="2" t="inlineStr">
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>Color System</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E149" s="2" t="inlineStr">
+      <c r="E150" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift exists; its detail modal is open.</t>
         </is>
       </c>
-      <c r="F149" s="2" t="inlineStr">
+      <c r="F150" s="2" t="inlineStr">
         <is>
           <t>1. Open the color picker in the modal.
 2. Choose a non-default color.
 3. Look at the block on the grid.</t>
         </is>
       </c>
-      <c r="G149" s="2" t="inlineStr">
+      <c r="G150" s="2" t="inlineStr">
         <is>
           <t>1. The shift's block re-renders in the chosen color.
 2. The color provides three consistent tones: background fill, text color, and accent (left border).
 3. Colors carry no fixed meaning - they are free choice beyond the two defaults (blue shift / grey event).</t>
         </is>
       </c>
-      <c r="H149" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §10, §4.9 (Color picker)</t>
-        </is>
-      </c>
-      <c r="I149" s="2" t="inlineStr"/>
-      <c r="J149" s="2" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§10, §4.9 (Color picker))</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
         <is>
           <t>Color labels are editable per shop</t>
         </is>
       </c>
-      <c r="B150" s="2" t="inlineStr">
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>Color System</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D150" s="2" t="inlineStr">
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E150" s="2" t="inlineStr">
+      <c r="E151" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shift's or event's color picker is open.</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr">
+      <c r="F151" s="2" t="inlineStr">
         <is>
           <t>1. Find the editable label of one color in the picker.
 2. Rename it (for example to 'ZZAUTOTEST Rush').
@@ -7793,50 +7843,479 @@
 4. Restore the original label.</t>
         </is>
       </c>
-      <c r="G150" s="2" t="inlineStr">
+      <c r="G151" s="2" t="inlineStr">
         <is>
           <t>1. Each color's label can be edited.
 2. The renamed label shows for the whole shop - the same picker opened elsewhere shows 'ZZAUTOTEST Rush'.
 3. Shifts and events share the same custom palette with the same labels.</t>
         </is>
       </c>
-      <c r="H150" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §10 (Color labels are editable per shop), §4.10 (shared picker)</t>
-        </is>
-      </c>
-      <c r="I150" s="2" t="inlineStr"/>
-      <c r="J150" s="2" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>SV-8700 (§10 (Color labels are editable per shop), §4.10 (shared picker))</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr"/>
+      <c r="J151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>Edit Location has a 'Set business hours for this shop' toggle, off by default</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to the ShopView App with access to location settings.
+2. You open the Edit Location screen for a shop.</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Edit Location screen.
+2. Find the business hours setting and read its default state.
+3. Turn the 'Set business hours for this shop' toggle ON.</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>1. Edit Location shows a toggle labelled 'Set business hours for this shop'.
+2. The toggle is OFF by default (no business hours set).
+3. Turning it ON reveals a per-day working-hours editor for the shop.</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - business hours toggle)</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>Edit Location shows a per-day (Mon-Sun) From-To business-hours editor</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>1. You are on the Edit Location screen.
+2. The 'Set business hours for this shop' toggle is ON.</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>1. Read the per-day rows shown when business hours are ON.
+2. Set a From time and a To time for one day (for example Monday).
+3. Save the location settings.</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>1. There is one row per day of the week, Monday through Sunday.
+2. Each day has a From time and a To time you can set.
+3. The saved shop business hours are used by the Schedule (start-time hierarchy, before/after-hours conflicts, business-hours shading).</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - per-day From/To editor)</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr"/>
+      <c r="J153" s="2" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Edit Staff has a 'Set custom hours for this technician' toggle, off by default</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in with access to staff settings.
+2. You open the Edit Staff Member screen for a technician.</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Edit Staff Member screen for a technician.
+2. Find the custom-hours setting and read its default state.
+3. Turn the 'Set custom hours for this technician' toggle ON.</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>1. Edit Staff Member shows a toggle labelled 'Set custom hours for this technician'.
+2. The toggle is OFF by default (no custom hours set).
+3. Turning it ON reveals a per-day working-hours editor for that technician.</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - technician custom-hours toggle)</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>A technician with no custom hours inherits the shop business hours</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>1. The shop has business hours set (/02).
+2. A technician has the 'Set custom hours for this technician' toggle OFF.</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>1. Confirm the technician has no custom hours set.
+2. Schedule a shift for that technician and check start-time defaults / before-after-hours conflicts against the shop business hours.</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>1. With no custom hours, the technician's working hours fall back to the shop business hours.
+2. Start-time defaults and before/after-hours conflict checks for that technician use the shop business hours.</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - inherit shop hours when no custom hours)</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr"/>
+      <c r="J155" s="2" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>'Add hours' appends a removable second range for split shifts, starting empty</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>1. You are in the per-day working-hours editor (location or technician) with a day's first range set.</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>1. On one day, click 'Add hours'.
+2. Read the new range that appears.
+3. Set the second range, then remove it.</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>1. 'Add hours' appends an additional From-To range to that day (to support split shifts).
+2. The added range starts empty (no From/To pre-filled).
+3. Each added range can be removed individually.</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - Add hours split shifts)</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>Overlapping hour ranges flag red with a message and disable Save</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>1. You are in the per-day working-hours editor with at least two ranges on one day.</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>1. Set two ranges on the same day so their times overlap.
+2. Look at the offending range and the Save button.</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>1. The offending (overlapping) range is flagged in red.
+2. An inline message reads 'These hours overlap. Adjust the times so they don't conflict.'
+3. Save is disabled while the overlap exists.</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - overlap validation)</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr"/>
+      <c r="J157" s="2" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>Incomplete hour rows (empty From or To) are ignored by the overlap check</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Working Hours Settings</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>1. You are in the per-day working-hours editor with one complete range and one empty added range.</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>1. On one day, add a range but leave its From and/or To empty.
+2. Look at the validation state and the Save button.</t>
+        </is>
+      </c>
+      <c r="G158" s="2" t="inlineStr">
+        <is>
+          <t>1. The incomplete row (empty From/To) is ignored by the overlap check - it does not raise the overlap error.
+2. Save is not blocked by an incomplete row on its own (only genuine overlaps disable Save).</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>SV-8699 (§4.2 Working Hours - incomplete rows ignored by overlap check)</t>
+        </is>
+      </c>
+      <c r="I158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>Week Export opens a printable Department-by-Technician week grid</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Week Export and Printing</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>1. You are on the Schedule screen in Week view with some shifts scheduled.
+2. Your role has Schedule: View.</t>
+        </is>
+      </c>
+      <c r="F159" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the Week Export / Print action for the current week.
+2. Read the exported / printable layout.</t>
+        </is>
+      </c>
+      <c r="G159" s="2" t="inlineStr">
+        <is>
+          <t>1. A printable week view opens laid out as a Department-by-Technician grid for the week.
+2. It is formatted for printing (a clean page layout, without the interactive grid controls).</t>
+        </is>
+      </c>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (design Week Export - V1 scope pending Branko)</t>
+        </is>
+      </c>
+      <c r="I159" s="2" t="inlineStr"/>
+      <c r="J159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>Exported week view lists each department with its technicians and shifts</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Week Export and Printing</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>1. You have opened the Week Export / Print view for a week that has shifts.</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>1. Read the exported week view.
+2. Check the department grouping, the technician rows, and the shifts shown per day.</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>1. The exported view groups technicians by department, with department headers.
+2. Each technician's shifts for the week appear in the correct day columns.
+3. The week's date range is shown.</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (design Week Export - V1 scope pending Branko)</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr"/>
+      <c r="J160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
         <is>
           <t>Schedule: View grants the full read experience - page, all three views, mini calendar, search, filter, tooltips, read-only modals</t>
         </is>
       </c>
-      <c r="B151" s="2" t="inlineStr">
+      <c r="B161" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C151" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D151" s="2" t="inlineStr">
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E151" s="2" t="inlineStr">
+      <c r="E161" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: View but NOT Edit (assign a suitable system role or a purpose-made custom role; restore after).
 2. Shifts and events exist on the grid, created by an Edit-capable user.
 3. You are signed in AS that View-only user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F151" s="2" t="inlineStr">
+      <c r="F161" s="2" t="inlineStr">
         <is>
           <t>1. Open the Schedule page.
 2. Switch between Day, Week, and Month.
@@ -7844,7 +8323,7 @@
 4. Hover a shift for its tooltip, then click it to open the detail modal.</t>
         </is>
       </c>
-      <c r="G151" s="2" t="inlineStr">
+      <c r="G161" s="2" t="inlineStr">
         <is>
           <t>1. The Schedule page opens and all three views work.
 2. The mini calendar, search, and filters all work.
@@ -7852,43 +8331,43 @@
 4. Tooltips show on hover, and the shift/event detail modals open in read-only mode.</t>
         </is>
       </c>
-      <c r="H151" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (Schedule: View), §14.3</t>
-        </is>
-      </c>
-      <c r="I151" s="2" t="inlineStr"/>
-      <c r="J151" s="2" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.1 (Schedule: View), §14.3)</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr"/>
+      <c r="J161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
         <is>
           <t>View-only: every editing affordance is hidden or disabled</t>
         </is>
       </c>
-      <c r="B152" s="2" t="inlineStr">
+      <c r="B162" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C152" s="2" t="inlineStr">
+      <c r="C162" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D152" s="2" t="inlineStr">
+      <c r="D162" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E152" s="2" t="inlineStr">
+      <c r="E162" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: View but NOT Edit.
 2. Shifts, a series, and events exist on the grid.
 3. You are signed in AS that View-only user on a desktop browser, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F152" s="2" t="inlineStr">
+      <c r="F162" s="2" t="inlineStr">
         <is>
           <t>1. Look for drag handles on sidebar lines and try to drag a work order card onto the grid.
 2. Try dragging an existing shift block (move/reassign) and look for resize handles in day view.
@@ -7896,7 +8375,7 @@
 4. Open a shift's detail modal and inspect its fields and actions.</t>
         </is>
       </c>
-      <c r="G152" s="2" t="inlineStr">
+      <c r="G162" s="2" t="inlineStr">
         <is>
           <t>1. No drag handles are offered and nothing can be dragged from the sidebar onto the grid.
 2. Shift blocks cannot be moved or resized - no drop targets or resize handles appear.
@@ -7904,89 +8383,89 @@
 4. In the modal, edit fields are hidden or disabled, and the reassign and delete actions are absent.</t>
         </is>
       </c>
-      <c r="H152" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (Schedule: View - editing affordances hidden or disabled)</t>
-        </is>
-      </c>
-      <c r="I152" s="2" t="inlineStr"/>
-      <c r="J152" s="2" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" s="2" t="inlineStr">
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.1 (Schedule: View - editing affordances hidden or disabled))</t>
+        </is>
+      </c>
+      <c r="I162" s="2" t="inlineStr"/>
+      <c r="J162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
         <is>
           <t>With Schedule: View OFF, the Schedule top-level nav item is hidden entirely</t>
         </is>
       </c>
-      <c r="B153" s="2" t="inlineStr">
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C153" s="2" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D153" s="2" t="inlineStr">
+      <c r="D163" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E153" s="2" t="inlineStr">
+      <c r="E163" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: View OFF (no Schedule permission).
 2. You are signed in AS that user on a desktop browser.</t>
         </is>
       </c>
-      <c r="F153" s="2" t="inlineStr">
+      <c r="F163" s="2" t="inlineStr">
         <is>
           <t>1. Look at the app's main navigation.
 2. Search the nav for any Schedule entry.</t>
         </is>
       </c>
-      <c r="G153" s="2" t="inlineStr">
+      <c r="G163" s="2" t="inlineStr">
         <is>
           <t>1. The Schedule top-level nav item is not shown at all.
 2. The rest of the app works normally for the role.</t>
         </is>
       </c>
-      <c r="H153" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (When Schedule: View is OFF)</t>
-        </is>
-      </c>
-      <c r="I153" s="2" t="inlineStr"/>
-      <c r="J153" s="2" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="2" t="inlineStr">
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.1 (When Schedule: View is OFF))</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr"/>
+      <c r="J163" s="2" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>Schedule: Edit unlocks all creation and modification interactions</t>
         </is>
       </c>
-      <c r="B154" s="2" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C154" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D154" s="2" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E154" s="2" t="inlineStr">
+      <c r="E164" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: Edit (and View) but NOT Delete.
 2. Work orders with approved lines exist; you are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F154" s="2" t="inlineStr">
+      <c r="F164" s="2" t="inlineStr">
         <is>
           <t>1. Drag a work order from the sidebar onto a technician cell and complete the scope picker (and spread modal for a large job).
 2. Right-click a cell and create an event via 'New Event'; in day view, click empty space to create.
@@ -7995,7 +8474,7 @@
 5. Edit fields in the shift and event detail modals.</t>
         </is>
       </c>
-      <c r="G154" s="2" t="inlineStr">
+      <c r="G164" s="2" t="inlineStr">
         <is>
           <t>1. Drag-and-drop from the sidebar, the scope picker, and the spread modal all work.
 2. Shift and event creation works, including via the right-click context menu and day-view click-to-create.
@@ -8004,100 +8483,100 @@
 5. Modal fields are editable and save.</t>
         </is>
       </c>
-      <c r="H154" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (Schedule: Edit)</t>
-        </is>
-      </c>
-      <c r="I154" s="2" t="inlineStr"/>
-      <c r="J154" s="2" t="inlineStr"/>
-    </row>
-    <row r="155">
-      <c r="A155" s="2" t="inlineStr">
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.1 (Schedule: Edit))</t>
+        </is>
+      </c>
+      <c r="I164" s="2" t="inlineStr"/>
+      <c r="J164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
         <is>
           <t>Edit without Delete: the user can create and modify but cannot remove - delete action and trash icon hidden</t>
         </is>
       </c>
-      <c r="B155" s="2" t="inlineStr">
+      <c r="B165" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C155" s="2" t="inlineStr">
+      <c r="C165" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D155" s="2" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E155" s="2" t="inlineStr">
+      <c r="E165" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: Edit but NOT Delete.
 2. A shift, a series, and an event exist (some created by this user).
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F155" s="2" t="inlineStr">
+      <c r="F165" s="2" t="inlineStr">
         <is>
           <t>1. Open a shift's detail modal and look for the delete action / trash icon.
 2. Open an event's modal and look for a delete action.
 3. Try to find ANY way to remove a shift or event.</t>
         </is>
       </c>
-      <c r="G155" s="2" t="inlineStr">
+      <c r="G165" s="2" t="inlineStr">
         <is>
           <t>1. The delete action and the trash icon are hidden in the shift modal.
 2. Events likewise offer no delete.
 3. No path exists to remove shifts or events - while creating and modifying still work.</t>
         </is>
       </c>
-      <c r="H155" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (Schedule: Delete - without it)</t>
-        </is>
-      </c>
-      <c r="I155" s="2" t="inlineStr"/>
-      <c r="J155" s="2" t="inlineStr"/>
-    </row>
-    <row r="156">
-      <c r="A156" s="2" t="inlineStr">
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.1 (Schedule: Delete - without it))</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr"/>
+      <c r="J165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
         <is>
           <t>Schedule: Delete unlocks deleting shifts and events, including the three series-aware scopes</t>
         </is>
       </c>
-      <c r="B156" s="2" t="inlineStr">
+      <c r="B166" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C156" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D156" s="2" t="inlineStr">
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E156" s="2" t="inlineStr">
+      <c r="E166" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule: Delete.
 2. A standalone shift, a series, and an event exist.
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F156" s="2" t="inlineStr">
+      <c r="F166" s="2" t="inlineStr">
         <is>
           <t>1. Delete the standalone shift.
 2. Delete a series shift and read the scope options.
 3. Delete the event.</t>
         </is>
       </c>
-      <c r="G156" s="2" t="inlineStr">
+      <c r="G166" s="2" t="inlineStr">
         <is>
           <t>1. The delete action is available and works for shifts.
 2. Series deletion offers its scopes (this shift / this and after / whole series).
@@ -8105,389 +8584,389 @@
 4. Undo toasts appear (restore the items via Undo to clean up).</t>
         </is>
       </c>
-      <c r="H156" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.1 (Schedule: Delete)</t>
-        </is>
-      </c>
-      <c r="I156" s="2" t="inlineStr"/>
-      <c r="J156" s="2" t="inlineStr"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="2" t="inlineStr">
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.1 (Schedule: Delete))</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr"/>
+      <c r="J166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
         <is>
           <t>The permission tiers depend on each other: Delete requires Edit, and Edit requires View</t>
         </is>
       </c>
-      <c r="B157" s="2" t="inlineStr">
+      <c r="B167" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C157" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D157" s="2" t="inlineStr">
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E157" s="2" t="inlineStr">
+      <c r="E167" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in as an admin who can edit custom roles.
 2. A ZZAUTOTEST custom role exists (create one; delete after).</t>
         </is>
       </c>
-      <c r="F157" s="2" t="inlineStr">
+      <c r="F167" s="2" t="inlineStr">
         <is>
           <t>1. In the role's Schedule permissions, try to enable Edit while View is off.
 2. Try to enable Delete while Edit is off.
 3. Enable View, then Edit, then Delete in order.</t>
         </is>
       </c>
-      <c r="G157" s="2" t="inlineStr">
+      <c r="G167" s="2" t="inlineStr">
         <is>
           <t>1. Edit cannot be granted without View (the admin UI enforces or auto-selects the dependency).
 2. Delete cannot be granted without Edit.
 3. The three tiers can be enabled in dependency order, so each higher level always includes the ones beneath it (Delete includes Edit, and Edit includes View).</t>
         </is>
       </c>
-      <c r="H157" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14 (Delete requires Edit and Edit requires View)</t>
-        </is>
-      </c>
-      <c r="I157" s="2" t="inlineStr"/>
-      <c r="J157" s="2" t="inlineStr"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="2" t="inlineStr">
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14 (Delete requires Edit and Edit requires View))</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr"/>
+      <c r="J167" s="2" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
         <is>
           <t>Schedule access without Work Orders: View - sidebar hides the WO list and drill-down; mini calendar stays; grid shifts remain usable</t>
         </is>
       </c>
-      <c r="B158" s="2" t="inlineStr">
+      <c r="B168" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C158" s="2" t="inlineStr">
+      <c r="C168" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D158" s="2" t="inlineStr">
+      <c r="D168" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E158" s="2" t="inlineStr">
+      <c r="E168" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule access but Work Orders: View OFF.
 2. Shifts already exist on the grid.
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F158" s="2" t="inlineStr">
+      <c r="F168" s="2" t="inlineStr">
         <is>
           <t>1. Look at the left sidebar.
 2. Interact with the shifts already on the grid (hover, open modal, and - if the role has Edit - move one).
 3. Try to find any way to drag a new work order onto the grid.</t>
         </is>
       </c>
-      <c r="G158" s="2" t="inlineStr">
+      <c r="G168" s="2" t="inlineStr">
         <is>
           <t>1. The sidebar hides the work order list and the line drill-down; the mini calendar remains available.
 2. Shifts already on the grid can still be viewed and interacted with per the role's Schedule tier.
 3. New work orders cannot be dragged on - the WO list is simply not visible.</t>
         </is>
       </c>
-      <c r="H158" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.2</t>
-        </is>
-      </c>
-      <c r="I158" s="2" t="inlineStr"/>
-      <c r="J158" s="2" t="inlineStr"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="2" t="inlineStr">
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>SV-8687 (§14.2)</t>
+        </is>
+      </c>
+      <c r="I168" s="2" t="inlineStr"/>
+      <c r="J168" s="2" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
         <is>
           <t>No own-only restriction: every Schedule: View user sees ALL technicians' shifts and events</t>
         </is>
       </c>
-      <c r="B159" s="2" t="inlineStr">
+      <c r="B169" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D159" s="2" t="inlineStr">
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E159" s="2" t="inlineStr">
+      <c r="E169" s="2" t="inlineStr">
         <is>
           <t>1. Shifts and events exist for SEVERAL different technicians.
 2. A test user with a low-tier View-only role exists (and is themselves one of the technicians).
 3. You are signed in AS that user, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F159" s="2" t="inlineStr">
+      <c r="F169" s="2" t="inlineStr">
         <is>
           <t>1. Read the grid across all departments and technicians.
 2. Check 'My Shifts' in 'Filter and Display' is OFF (default).</t>
         </is>
       </c>
-      <c r="G159" s="2" t="inlineStr">
+      <c r="G169" s="2" t="inlineStr">
         <is>
           <t>1. The user sees ALL technicians' shifts and events, not only their own - there is no role-based 'own shifts only' restriction.
 2. 'My Shifts' exists only as an optional personal convenience filter (off by default), not a security boundary.</t>
         </is>
       </c>
-      <c r="H159" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.3</t>
-        </is>
-      </c>
-      <c r="I159" s="2" t="inlineStr"/>
-      <c r="J159" s="2" t="inlineStr"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="2" t="inlineStr">
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>SV-8685 (§14.3)</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr"/>
+      <c r="J169" s="2" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
         <is>
           <t>Grid rows are department-based: any staff member in a visible department appears as a row, regardless of role</t>
         </is>
       </c>
-      <c r="B160" s="2" t="inlineStr">
+      <c r="B170" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C160" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D160" s="2" t="inlineStr">
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E160" s="2" t="inlineStr">
+      <c r="E170" s="2" t="inlineStr">
         <is>
           <t>1. A staff member with a NON-technician role (for example Office) is assigned to a department that is visible on the schedule (set up; restore after).
 2. Another staff member has NO department assignment.
 3. You are signed in on a desktop browser, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F160" s="2" t="inlineStr">
+      <c r="F170" s="2" t="inlineStr">
         <is>
           <t>1. Look for the department-assigned Office staff member among the grid rows.
 2. Look for the staff member with no department.</t>
         </is>
       </c>
-      <c r="G160" s="2" t="inlineStr">
+      <c r="G170" s="2" t="inlineStr">
         <is>
           <t>1. The department-assigned staff member appears as a technician row - row presence is controlled by the department on the staff record, NOT by role permission.
 2. The staff member without a department does not appear as a row.</t>
         </is>
       </c>
-      <c r="H160" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.4</t>
-        </is>
-      </c>
-      <c r="I160" s="2" t="inlineStr"/>
-      <c r="J160" s="2" t="inlineStr"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="2" t="inlineStr">
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>SV-8686 (§14.4)</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr"/>
+      <c r="J170" s="2" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
         <is>
           <t>Clocking into work order line tasks is gated by the staff record's 'Time Clock' setting, not the permission model</t>
         </is>
       </c>
-      <c r="B161" s="2" t="inlineStr">
+      <c r="B171" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C161" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D161" s="2" t="inlineStr">
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E161" s="2" t="inlineStr">
+      <c r="E171" s="2" t="inlineStr">
         <is>
           <t>1. Two staff members exist: one with the 'Time Clock' setting ON on their staff record, one with it OFF (set up; restore after).
 2. Both appear as schedule rows and have shifts on work order lines.</t>
         </is>
       </c>
-      <c r="F161" s="2" t="inlineStr">
+      <c r="F171" s="2" t="inlineStr">
         <is>
           <t>1. As (or with) the Time-Clock-ON staff member, attempt to clock into their work order line task.
 2. As (or with) the Time-Clock-OFF staff member, attempt the same.</t>
         </is>
       </c>
-      <c r="G161" s="2" t="inlineStr">
+      <c r="G171" s="2" t="inlineStr">
         <is>
           <t>1. The Time-Clock-ON staff member can clock in.
 2. The Time-Clock-OFF staff member cannot - the ability is controlled by the staff-record setting, not by the Schedule permission tier.</t>
         </is>
       </c>
-      <c r="H161" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.4 (Time Clock setting)</t>
-        </is>
-      </c>
-      <c r="I161" s="2" t="inlineStr"/>
-      <c r="J161" s="2" t="inlineStr"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="2" t="inlineStr">
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>SV-8686 (§14.4 (Time Clock setting))</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr"/>
+      <c r="J171" s="2" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
         <is>
           <t>With Work Orders: View OFF, work-order-derived details on shifts (customer, lines, money fields) are hidden or masked</t>
         </is>
       </c>
-      <c r="B162" s="2" t="inlineStr">
+      <c r="B172" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
+      <c r="C172" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D162" s="2" t="inlineStr">
+      <c r="D172" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E162" s="2" t="inlineStr">
+      <c r="E172" s="2" t="inlineStr">
         <is>
           <t>1. A test user's role has Schedule access but Work Orders: View OFF (assign a suitable role; restore after).
 2. Shifts already exist on the grid, created by a fully-permissioned user, for units that have customers, scheduled lines, and a VIN.
 3. You are signed in AS that user on a desktop browser, on the Schedule page.</t>
         </is>
       </c>
-      <c r="F162" s="2" t="inlineStr">
+      <c r="F172" s="2" t="inlineStr">
         <is>
           <t>1. Look at a shift block on the grid and read its text lines.
 2. Hover the shift for its tooltip.
 3. Open the shift's detail modal and read the work-order-derived fields.</t>
         </is>
       </c>
-      <c r="G162" s="2" t="inlineStr">
+      <c r="G172" s="2" t="inlineStr">
         <is>
           <t>1. Work-order-derived details (customer, the scheduled line list, and any money-bearing fields) are hidden or masked wherever they would normally appear - on the block, in the tooltip, and in the modal.
 2. The schedule structure itself (the shift's day, time, and technician) stays visible so the grid remains usable.
 3. This extends the sidebar behavior (the work order list and drill-down are hidden) to the work-order data surfaced on the shifts themselves.</t>
         </is>
       </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §14.2 (Work Orders: View dependency)</t>
-        </is>
-      </c>
-      <c r="I162" s="2" t="inlineStr"/>
-      <c r="J162" s="2" t="inlineStr"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="2" t="inlineStr">
+      <c r="H172" s="2" t="inlineStr">
+        <is>
+          <t>SV-8687 (§14.2 (Work Orders: View dependency))</t>
+        </is>
+      </c>
+      <c r="I172" s="2" t="inlineStr"/>
+      <c r="J172" s="2" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
         <is>
           <t>Planned hours across technicians may exceed the estimate - accepted without error</t>
         </is>
       </c>
-      <c r="B163" s="2" t="inlineStr">
+      <c r="B173" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D163" s="2" t="inlineStr">
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E163" s="2" t="inlineStr">
+      <c r="E173" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A work order line with a 40h estimate exists.</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr">
+      <c r="F173" s="2" t="inlineStr">
         <is>
           <t>1. Spread the full estimate onto technician A.
 2. Spread the full estimate of the SAME work order onto technician B.
 3. Look for any warning or error about exceeding the estimate.</t>
         </is>
       </c>
-      <c r="G163" s="2" t="inlineStr">
+      <c r="G173" s="2" t="inlineStr">
         <is>
           <t>1. Both series are created - 80 planned hours against a 40h estimate is accepted.
 2. No error or blocking warning appears - this is expected behavior because progress is driven by clocked-in time, and scheduled hours, the estimate, and actual hours are three separate quantities that are not forced to reconcile.</t>
         </is>
       </c>
-      <c r="H163" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §12, §4.5</t>
-        </is>
-      </c>
-      <c r="I163" s="2" t="inlineStr"/>
-      <c r="J163" s="2" t="inlineStr"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="2" t="inlineStr">
+      <c r="H173" s="2" t="inlineStr">
+        <is>
+          <t>SV-8691 (§12, §4.5)</t>
+        </is>
+      </c>
+      <c r="I173" s="2" t="inlineStr"/>
+      <c r="J173" s="2" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
         <is>
           <t>Below 960px the grid scrolls horizontally, and the sidebar collapses on narrow viewports</t>
         </is>
       </c>
-      <c r="B164" s="2" t="inlineStr">
+      <c r="B174" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D164" s="2" t="inlineStr">
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E164" s="2" t="inlineStr">
+      <c r="E174" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
 2. You are on the Schedule page in week view with shifts visible.</t>
         </is>
       </c>
-      <c r="F164" s="2" t="inlineStr">
+      <c r="F174" s="2" t="inlineStr">
         <is>
           <t>1. Resize the browser window to just under 960px wide.
 2. Try to reach the right-hand days of the grid.
 3. Narrow the window further and watch the sidebar.</t>
         </is>
       </c>
-      <c r="G164" s="2" t="inlineStr">
+      <c r="G174" s="2" t="inlineStr">
         <is>
           <t>1. Below the 960px minimum supported width, the grid scrolls horizontally rather than breaking.
 2. All days remain reachable by horizontal scroll.
@@ -8495,210 +8974,210 @@
 4. No content becomes permanently unreachable and nothing errors.</t>
         </is>
       </c>
-      <c r="H164" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §11 (Responsiveness)</t>
-        </is>
-      </c>
-      <c r="I164" s="2" t="inlineStr"/>
-      <c r="J164" s="2" t="inlineStr"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="2" t="inlineStr">
+      <c r="H174" s="2" t="inlineStr">
+        <is>
+          <t>SV-8686 (§11 (Responsiveness))</t>
+        </is>
+      </c>
+      <c r="I174" s="2" t="inlineStr"/>
+      <c r="J174" s="2" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
         <is>
           <t>The sidebar work order list and line drill-down stay smooth with 50+ items</t>
         </is>
       </c>
-      <c r="B165" s="2" t="inlineStr">
+      <c r="B175" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D165" s="2" t="inlineStr">
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E165" s="2" t="inlineStr">
+      <c r="E175" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
 2. 50 or more open work orders exist (seed ZZAUTOTEST orders if the environment lacks them), including one order with many approved lines.
 3. You are on the Schedule page.</t>
         </is>
       </c>
-      <c r="F165" s="2" t="inlineStr">
+      <c r="F175" s="2" t="inlineStr">
         <is>
           <t>1. Scroll the full work order list top to bottom quickly.
 2. Open the many-line order's drill-down and scroll it.
 3. Type in the search while the long list is shown.</t>
         </is>
       </c>
-      <c r="G165" s="2" t="inlineStr">
+      <c r="G175" s="2" t="inlineStr">
         <is>
           <t>1. Scrolling stays smooth with no long freezes or blank stretches that fail to fill in (the list virtualizes at 50+ items).
 2. The drill-down behaves the same with many lines.
 3. Search stays responsive on the long list.</t>
         </is>
       </c>
-      <c r="H165" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §11 (Performance - virtualization)</t>
-        </is>
-      </c>
-      <c r="I165" s="2" t="inlineStr"/>
-      <c r="J165" s="2" t="inlineStr"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="2" t="inlineStr">
+      <c r="H175" s="2" t="inlineStr">
+        <is>
+          <t>SV-8686 (§11 (Performance - virtualization))</t>
+        </is>
+      </c>
+      <c r="I175" s="2" t="inlineStr"/>
+      <c r="J175" s="2" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
         <is>
           <t>The grid renders smoothly at full load - 15 technicians × 7 days with several shifts per cell</t>
         </is>
       </c>
-      <c r="B166" s="2" t="inlineStr">
+      <c r="B176" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D166" s="2" t="inlineStr">
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E166" s="2" t="inlineStr">
+      <c r="E176" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
 2. The schedule is loaded to roughly the spec's stated scale: around 15 technician rows across a week with several shifts per cell (seed ZZAUTOTEST shifts as needed).
 3. You are on the Schedule page in week view.</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr">
+      <c r="F176" s="2" t="inlineStr">
         <is>
           <t>1. Scroll the grid vertically and horizontally.
 2. Switch between Day, Week, and Month.
 3. Hover several blocks and open/close a modal.</t>
         </is>
       </c>
-      <c r="G166" s="2" t="inlineStr">
+      <c r="G176" s="2" t="inlineStr">
         <is>
           <t>1. The grid renders and scrolls smoothly at this scale.
 2. View switches complete without long hangs.
 3. Tooltips and modals stay responsive.</t>
         </is>
       </c>
-      <c r="H166" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §11 (Performance)</t>
-        </is>
-      </c>
-      <c r="I166" s="2" t="inlineStr"/>
-      <c r="J166" s="2" t="inlineStr"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="2" t="inlineStr">
-        <is>
-          <t>Shop closures block the spread step from placing shifts on those days</t>
-        </is>
-      </c>
-      <c r="B167" s="2" t="inlineStr">
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>SV-8686 (§11 (Performance))</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr"/>
+      <c r="J176" s="2" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>Shop closures do NOT block spread in V1 - shifts can land on closure days</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C167" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D167" s="2" t="inlineStr">
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E167" s="2" t="inlineStr">
+      <c r="E177" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A shop closure (holiday/inventory day) is defined at the shop level on a working weekday inside the planned spread window (set it up; remove after).
 3. A large job (multi-day scope) is ready to spread.</t>
         </is>
       </c>
-      <c r="F167" s="2" t="inlineStr">
-        <is>
-          <t>1. Open the spread step across the window containing the closure.
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>1. Open the spread step across a window that contains a shop closure day.
 2. Expand the preview and find the closure day.
 3. Confirm the spread and check the grid.</t>
         </is>
       </c>
-      <c r="G167" s="2" t="inlineStr">
-        <is>
-          <t>1. The preview shows the closure day struck through with its reason.
-2. No shift is placed on the closure day - the series flows around it.
-3. The series' end date extends accordingly (the skipped day's hours land on later working days).</t>
-        </is>
-      </c>
-      <c r="H167" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §12 (Shop closures), §4.5</t>
-        </is>
-      </c>
-      <c r="I167" s="2" t="inlineStr"/>
-      <c r="J167" s="2" t="inlineStr"/>
-    </row>
-    <row r="168">
-      <c r="A168" s="2" t="inlineStr">
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>1. The closure day is NOT struck through or skipped by the spread in V1.
+2. A shift CAN be placed on the shop closure day (only weekend days with no business hours are skipped).
+3. The end date follows the normal daily distribution - no extra day is added for the closure.</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>SV-8691 (§12 (Shop closures), §4.5)</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr"/>
+      <c r="J177" s="2" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
         <is>
           <t>Scheduled hours, the estimate, and actual (clocked) hours are three separate quantities that are not forced to reconcile</t>
         </is>
       </c>
-      <c r="B168" s="2" t="inlineStr">
+      <c r="B178" s="2" t="inlineStr">
         <is>
           <t>Edge Cases and Responsiveness</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E168" s="2" t="inlineStr">
+      <c r="E178" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser with Schedule: Edit.
 2. A line has estimate 10h; a technician has 6h scheduled against it and some different amount of time actually clocked (seed what is possible).</t>
         </is>
       </c>
-      <c r="F168" s="2" t="inlineStr">
+      <c r="F178" s="2" t="inlineStr">
         <is>
           <t>1. Open the shift's detail modal.
 2. Compare the scheduled hours, the estimate, and the logged/actual time.</t>
         </is>
       </c>
-      <c r="G168" s="2" t="inlineStr">
+      <c r="G178" s="2" t="inlineStr">
         <is>
           <t>1. All three quantities are shown/derivable and may differ from one another.
 2. Nothing forces them to match - no error, no auto-correction (progress is driven by clocked-in time).</t>
         </is>
       </c>
-      <c r="H168" s="2" t="inlineStr">
-        <is>
-          <t>requirements.md §4.5 (three separate quantities), §12</t>
-        </is>
-      </c>
-      <c r="I168" s="2" t="inlineStr"/>
-      <c r="J168" s="2" t="inlineStr"/>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>SV-8691 (§4.5 (three separate quantities), §12)</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr"/>
+      <c r="J178" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Schedule currency: regenerate import + id-map to v30 (header sha256 == 6 peers, 0 shred, id-map 195/195 no blanks, refs match live)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/schedule-v1-testrail-import.xlsx
+++ b/testrail-import/schedule-v1-testrail-import.xlsx
@@ -528,8 +528,8 @@
 3. The left panel is the work order sidebar: a mini calendar at the top and a work order list beneath it.
 4. The main area is the schedule grid showing technician rows, with a toolbar above it.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3, §3.1, §3.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§3, §3.1, §3.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -585,8 +585,8 @@
 3. Month: the grid shows a compact calendar with per-day capacity bars and shift chips.
 4. The same shifts appear in all three views - each one drawn to suit that view: positioned on the hour line in Day, as a chip in the day column in Week, and as a compact chip in Month.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.2, §6), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§3.2, §6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -638,8 +638,8 @@
 2. Each department's technicians are listed beneath that department's header.
 3. Every staff member assigned to a visible department appears as a row, regardless of their role.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.2, §14.4), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§3.2, §14.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -692,8 +692,8 @@
 2. Expanding shows the technician rows again, unchanged.
 3. Other department groups are unaffected.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§3.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -742,8 +742,8 @@
           <t xml:space="preserve">1. No such toggle exists - the department-grouped rows are the only grid grouping.
 2. Department visibility is controlled only through the department toggles in the 'Filter &amp; display' dropdown.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§3.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -849,8 +849,8 @@
 2. Of the three buttons Day, Week and Month, the one that is switched on (highlighted) is Day.
 3. The grid shows the Day layout: a 24-hour timeline for each technician row, with shifts placed at their times.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the acceptance criterion of its story SV-8686, read on 11 August 2026, which states that when the schedule page loads the grid displays with day view as default. The Schedule specification version 27 does not say which view the page opens on, so this expectation comes from the story rather than the specification. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the acceptance criterion of its story SV-8686, read on 17 August 2026, which states that when the schedule page loads the grid displays with day view as default. The Schedule specification version 30 does not say which view the page opens on, so this expectation comes from the story rather than the specification.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -901,8 +901,8 @@
 2. The toolbar date label updates to the new range.
 3. The clicked date is highlighted as the selected date in the mini calendar.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1, §5.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1, §5.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -956,8 +956,8 @@
 2. Choosing a month shows that month in the mini calendar.
 3. The main grid can then be navigated by clicking a date in the newly shown month.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1010,8 +1010,8 @@
           <t xml:space="preserve">1. The calendar grid collapses (hides), leaving more room for the work order list below.
 2. Clicking again expands the calendar grid back.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1, §5.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1, §5.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1065,8 +1065,8 @@
 2. Today's date has its own distinct indicator, different from the selection.
 3. Hovering a week row highlights that whole week row.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1119,8 +1119,8 @@
 2. The list scrolls when there are more cards than fit.
 3. There are no Assigned/Unassigned tabs - assignment is available only as a filter behind the 'Filter' button.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1, §5.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1, §5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1289,8 +1289,8 @@
 2. Deleting characters widens the results again.
 3. With very many work orders, the list may load further results in pages as you scroll - that is expected, not a fault.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1344,8 +1344,8 @@
 2. The app does not error; the sidebar remains usable.
 3. Clearing the search restores the full list.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1513,8 +1513,8 @@
 2. Applying a filter narrows the flat card list.
 3. The 'Filters' button shows a badge with the number of active filters.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1569,8 +1569,8 @@
 2. Assigned: only work orders with a technician assigned remain.
 3. There are no Assigned/Unassigned tabs - this filter is the only assignment split.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.1, §3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.1, §3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1626,8 +1626,8 @@
 3. The card left-border colours of the remaining cards are consistent with that status.
 Note for the tester: this shop's schedule list only holds work orders in two statuses, Approved and Review, so most of the other choices correctly come back empty. An empty list for a status no work order is in is the right answer, not a fault.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1681,8 +1681,8 @@
           <t xml:space="preserve">1. The Priority group offers High, Medium, and Low.
 2. Only High-priority work orders remain in the list.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1725,7 +1725,7 @@
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Click 'Clear all'.
-2. Look at the list and the 'Filter' button.
+2. Look at the list and the 'Filters' button.
 </t>
         </is>
       </c>
@@ -1733,10 +1733,10 @@
         <is>
           <t xml:space="preserve">1. All applied filters are removed at once.
 2. The full work order list is shown again.
-3. The active-count badge on the 'Filter' button disappears (or shows zero).
----
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.1), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+3. The active-count badge on the 'Filters' button disappears (or shows zero).
+---
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1790,8 +1790,8 @@
           <t xml:space="preserve">1. The list shows only work orders that match BOTH the text search and the structured filter.
 2. Removing either the search text or the filter widens the list to the remaining condition.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§5.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1847,8 +1847,8 @@
 4. A back control is shown to return to the card list.
 5. Clicking back restores the work order card list.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1902,8 +1902,8 @@
 2. No line that has never been approved appears anywhere in the schedule sidebar - for example a line still sitting on an estimate, or one that was declined.
 3. The line count in the drill-down header matches the number of APPROVED lines on the work order - a line that was never approved is neither listed nor counted.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -1957,8 +1957,8 @@
 2. The current technician roster is shown as an avatar stack plus a count; there is no cap on how many technicians a line can have.
 3. Each line row has its own drag handle, so it can be dragged independently onto the grid.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1, §8.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1, §8.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2012,8 +2012,8 @@
 2. The line with a technician does not show the badge.
 3. After a technician is scheduled onto the badge-bearing line, the badge goes away.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2067,8 +2067,8 @@
           <t xml:space="preserve">1. Typing a line title narrows the list to matching lines.
 2. Typing the customer name returns no results - the line search matches line titles only (the list is already scoped to one work order, so customer/unit/WO fields are not searched).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2123,8 +2123,8 @@
 2. Unscheduled lists only the lines that have no shifts yet, and its count matches.
 3. All lists every approved line, and its count matches the drill-down header's line count.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§3.1, §5.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§3.1, §5.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2231,8 +2231,8 @@
 2. It offers 'Schedule whole work order' at the top, the individual line rows beneath, and a 'Select multiple' control.
 3. No shift is created until a scope is chosen.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.1, §4.3), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§4.1, §4.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2285,8 +2285,8 @@
 2. The block's last text line shows that line's name.
 3. The technician is added to that line's roster only (not to the order's other lines).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§4.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2391,8 +2391,8 @@
           <t xml:space="preserve">1. The shift is created straight away - the spread step does NOT appear.
 2. The shift sits on the dropped day only.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§4.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2444,8 +2444,8 @@
 2. A ghost block follows the drag showing the line name and its hours.
 3. Releasing outside any valid cell creates nothing.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2501,8 +2501,8 @@
 4. Dragging the same line onto a second technician adds that technician to the line's roster as well - the technician who was already there stays on it.
 5. Nothing asks you to swap or replace the technician who was already there, and no limit is reached on how many technicians a line can have.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§1.2, §4.3, §7), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§1.2, §4.3, §7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2552,13 +2552,9 @@
         <is>
           <t xml:space="preserve">1. The item can be placed onto a cell without holding a drag - clicking arms it, and clicking a cell places it.
 2. The result is the same as the equivalent drag-and-drop (scope picker / spread step rules apply the same way).
-What you should see today: there is no click alternative anywhere. The work order card in the left-hand panel carries no button that arms it for placing - not when the page loads, not when you rest the mouse on the card, and not inside the card's line list. The only way to place a job on the grid is to drag it. This is a known problem and it is already reported - see https://shopview.atlassian.net/browse/SV-8957. That ticket has been closed without the problem being fixed, so do not wait for a fix.
-- If you see exactly that, mark this test FAILED and do not raise anything new.
-- If it fails in a DIFFERENT way from what is described above, that is a NEW problem - please report it.
-- If it PASSES, the fix has shipped: tell the QA lead so the ticket can be closed and this note removed.
----
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7, §11), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: READY - EXPECT FAIL (SV-8957)
+---
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§7, §11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2613,10 +2609,10 @@
           <t xml:space="preserve">1. While the card is held over a day box, that day box shows it is a drop target.
 2. Releasing on the day box books the work order onto that day, exactly as dropping it does in Week view: because this work order has more than one line, the scope picker opens so you can choose the whole order, one line, or several lines.
 3. After you confirm a scope, a shift appears in that day box, and its start time comes from the usual order of preference - the technician's own working hours first, otherwise the shop's business hours, otherwise 7:00 AM.
-Please read before running this test: what should happen in MONTH view specifically has not been settled yet. The Schedule specification version 27 says that a work order is dragged from the sidebar onto a cell in the grid without naming which view, and the acceptance criterion of story SV-8688 names only Week view. The question has been put to the product owner on SV-8870 (https://shopview.atlassian.net/browse/SV-8870), together with the point that Month view invites the user to drag ("Nothing is scheduled in this range. Drag a work order from the list to book it."). Until the product owner answers, treat a failure here as already reported under SV-8870 - mark it FAILED and link SV-8870; do not raise a new ticket.
+Please read before running this test: what should happen in MONTH view specifically has not been settled yet. The Schedule specification version 30 says that a work order is dragged from the sidebar onto a cell in the grid without naming which view, and the acceptance criterion of story SV-8688 names only Week view. The question has been put to the product owner on SV-8870 (https://shopview.atlassian.net/browse/SV-8870), together with the point that Month view invites the user to drag ("Nothing is scheduled in this range. Drag a work order from the list to book it."). Until the product owner answers, treat a failure here as already reported under SV-8870 - mark it FAILED and link SV-8870; do not raise a new ticket.
 What was seen on the build checked: the card lifts and follows the mouse, but no day box shows as a drop target and releasing does nothing at all - no scope picker, no shift, no message. The same drag of the same work order in Week view does open the scope picker, so the difference is Month view itself.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.1, §4.2), read on 11 August 2026, which describe dragging a work order from the sidebar onto a cell in the grid and the order of preference for the start time. Neither that specification nor story SV-8688 says whether Month view accepts the drop, so that point is an open product-owner question rather than a settled requirement. Last checked against build v3.5-d122eef on 8/5/2026.
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§4.1, §4.2), read on 17 August 2026, which describe dragging a work order from the sidebar onto a cell in the grid and the order of preference for the start time. Neither that specification nor story SV-8688 says whether Month view accepts the drop, so that point is an open product-owner question rather than a settled requirement.
 AUTOMATION: HOLD - waiting on the product owner's answer, and the question has not been sent yet
 </t>
         </is>
@@ -2780,8 +2776,8 @@
 4. Each line row shows the line title and its estimated hours.
 5. Rows for lines that already have technicians show the current roster as an avatar stack plus count.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.3), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8689 and the Schedule specification version 30 (§4.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2834,8 +2830,8 @@
 2. The block's last text line reads 'N Lines' (with N = the line count).
 3. The technician is added to the roster of every one of those lines.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.3, §4.4), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8689 and the Schedule specification version 30 (§4.3, §4.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2887,8 +2883,8 @@
 2. The picker closes.
 3. The block's last text line shows the line's name.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.3), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8689 and the Schedule specification version 30 (§4.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2946,8 +2942,8 @@
 4. A 'Cancel' control leaves tick-box mode and returns you to the ordinary single-tap line list, without creating anything and without closing the picker.
 5. Confirming creates ONE shift covering exactly the ticked lines, and the technician is added to those lines' rosters only - not to the other lines.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.3), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: HOLD - not re-checked against the current build - it needs a drag that could not be completed
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8689 and the Schedule specification version 30 (§4.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -2999,8 +2995,8 @@
           <t xml:space="preserve">1. The shift starts at the technician's own configured start time (6:00 AM in the example), not the shop's business-hours start.
 Known issue on the build tested: the time this test talks about is stored correctly but the Schedule SHOWS it six hours later than it should be, so a 7:00 AM start reads 1:00 PM on screen. That is already raised with the developers as SV-8848 (https://shopview.atlassian.net/browse/SV-8848). Check the value is right by the rule this test describes, and ignore the six-hour display shift - do not raise a new ticket for it.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -3051,8 +3047,8 @@
         <is>
           <t xml:space="preserve">1. The shift starts at the shop's business-hours start time.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -3157,8 +3153,8 @@
 2. The start time aligns to the timeline position (see the 15-minute snapping case).
 Note for the tester: every time on the Schedule is currently shown six hours later than the time it was booked for. That is already reported as SV-8848 (https://shopview.atlassian.net/browse/SV-8848). Read the position on the timeline rather than the printed time, and do not raise it again.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -3173,7 +3169,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>Dropping onto the Unassigned row creates a shift with no technician</t>
+          <t>Dropping onto a department's unassigned lane creates a shift with no technician</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3200,24 +3196,24 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>1. Drag the line from the sidebar and drop it onto the grid's Unassigned row on a working day.
+          <t>1. Drag the line from the sidebar and drop it onto a department's unassigned lane (the department group header row) on a working day.
 2. Look at the created block and the line's roster.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. An unassigned shift is created in the Unassigned row for that day.
-2. It has no technician (and no technician is added to the line's roster by this drop).
-3. The block uses the same anatomy as a regular shift (customer, unit, line name / 'N Lines').
----
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2, §3.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+          <t xml:space="preserve">1. An unassigned shift is created in that department's unassigned lane. The department group header row doubles as the lane - there is no separate 'Unassigned' row.
+2. It has no technician, and no technician is added to the line's roster by this drop.
+3. The block renders as a fixed-width chip carrying its hours - it is not scaled to a duration, because no technician's hours have been applied to it yet.
+---
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-9234 and the Schedule specification version 30 (§4.2, §3.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>SV-8688 (§4.2 (Unassigned shifts),§3.2)</t>
+          <t>SV-9234 (§3.2 §4.2 unassigned lane on the department header row)</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -3226,7 +3222,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Unassigned shift start time uses business hours or the default</t>
+          <t>Unassigned shift start time uses business hours or the app-level default</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3254,22 +3250,23 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>1. Drop the line onto the Unassigned row.
+          <t>1. Drop the line onto a department's unassigned lane (the department group header row).
 2. Read the created shift's start time.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The unassigned shift starts at the shop's business-hours start (there is no technician whose hours could apply).
----
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+          <t xml:space="preserve">1. The unassigned shift takes its start time from the same rules as any shift, minus the technician level: the shop's business hours, or - if the shop has no business hours set - the app-level default of 7:00 AM.
+2. The day you dropped it on is recorded as the shift's target start date.
+---
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-9234 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>SV-8688 (§4.2)</t>
+          <t>SV-9234 (§4.2 unassigned shift start time)</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3605,8 +3602,8 @@
 4. Clicking 'Change scope' takes the modal back to the scope picker (step 1) without creating anything.
 5. Choosing a new scope updates the spread step's header and hours accordingly.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -3819,8 +3816,8 @@
 2. It can be changed; technician B's series then starts after A's series ends (sequential, not parallel).
 3. B's series is created from the adjusted start date onward.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: HOLD - not re-checked against the current build - it needs a drag that could not be completed
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -3982,8 +3979,8 @@
 3. Each daily shift keeps its own day and hours.
 4. A toast with Undo appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5, §4.6, §8.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: HOLD - not re-checked against the current build - it needs a drag that could not be completed
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5, §4.6, §8.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4035,8 +4032,8 @@
 2. There is no shared 'remaining hours' counter across technicians and no splitting of a shift.
 3. Planned hours across technicians may now exceed the estimate - this is expected and produces no error (progress is driven by clocked-in time).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5, §12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5, §12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4091,8 +4088,8 @@
 3. A single spread that would create more than 120 daily shifts is refused outright - no confirmation can override it, and no shifts are created for that attempt.
 4. No half-created series is left behind after a refused attempt.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5), read on 11 August 2026, with the specific limits above taken from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5), read on 17 August 2026, with the specific limits above taken from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4374,8 +4371,8 @@
 2. It is labeled once at the start (including the technician); later weeks show a faded 'continues'-style label instead of repeating the full label.
 3. Weekend columns inside the series are empty (no bar) when no business hours are set for those weekend days.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.6), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§4.6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4428,8 +4425,8 @@
 2. Chevrons at the banner's edges indicate the series continues beyond the visible week (both sides, on a middle week).
 3. A 'week N of M' cue shows the position within the series.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.6), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§4.6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4480,8 +4477,8 @@
           <t xml:space="preserve">1. The day shows a single time-positioned block (no spanning bar - only one day is visible).
 2. The block carries a cue in the spirit of 'part of an M-week job' indicating it belongs to a longer series.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.6), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§4.6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4534,8 +4531,8 @@
 2. The overlapping day is flagged as a Double-booked conflict, exactly as it would be for standalone shifts.
 3. The detail modal shows that single day's shift (its own day and hours) while indicating it belongs to the series.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.6, §8.2), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§4.6, §8.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4587,8 +4584,8 @@
 3. Last line: the name of the scheduled line.
 4. No work order number appears on the block.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.4), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8690 and the Schedule specification version 30 (§4.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4641,8 +4638,8 @@
 2. The subset block reads '2 Lines' - the block does not distinguish whole-order from subset beyond the count.
 3. Each detail modal lists exactly which lines the shift covers.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.4, §12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8690 and the Schedule specification version 30 (§4.4, §12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4694,8 +4691,8 @@
 2. The conflicted block shows the conflict (warning) icon on its first line - and that is the only icon that ever appears on a block.
 3. No scope icons distinguish whole-order from subset shifts.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.4), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8690 and the Schedule specification version 30 (§4.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4749,8 +4746,8 @@
 3. The row stays at its normal height.
 4. No conflict is flagged for back-to-back (non-intersecting) shifts.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.7, §12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8693 and the Schedule specification version 30 (§4.7, §12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4801,8 +4798,8 @@
 2. The row grows in height to fit the lanes.
 3. The overlap is also flagged as a Double-booked conflict (stacking reads as 'resolve me').
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.7, §4.11), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8693 and the Schedule specification version 30 (§4.7, §4.11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4856,8 +4853,8 @@
 4. You can tell the '+2 more' is something to click without relying on its colour: it carries the count as words you can read, and it is drawn as its own distinct shape - a small chip, pill or button - not just a differently coloured patch of the lane.
 5. The hidden shifts can be opened from that popover.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.7 Overlap and lane stacking and §11 Accessibility - the overflow uses shape), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8693 and the Schedule specification version 30 (§4.7 Overlap and lane stacking and §11 Accessibility - the overflow uses shape), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -4910,8 +4907,8 @@
 2. Week and month views reach the '+N more' overflow sooner than day view (their cells are narrower), but the same cap-and-overflow model applies.
 3. The overflow affordance opens the hidden-shifts popover in each view.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8693 and the Schedule specification version 30 (§4.7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5021,8 +5018,8 @@
           <t xml:space="preserve">1. In day view, the date/time header bar stays stuck to the top while the rows scroll beneath it - you always know which time column you are looking at.
 2. The same sticky-header behavior applies in week view.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.8), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8694 and the Schedule specification version 30 (§4.8), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5185,8 +5182,8 @@
 2. Its position matches the actual clock time.
 3. Hovering the now line while your pointer is over the grid shows a label (the current time).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.8), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8694 and the Schedule specification version 30 (§4.8), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5333,7 +5330,7 @@
       <c r="E90" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in on a desktop browser.
-2. A shift exists for a unit that has a VIN; the VIN toggle in 'Filter and Display' is OFF.
+2. A shift exists for a unit that has a VIN; the VIN toggle in 'Filter &amp; display' is OFF.
 3. You are on the Schedule page.</t>
         </is>
       </c>
@@ -5349,8 +5346,8 @@
 2. It shows the customer name, unit number, the VIN (below unit and asset), and the work order id.
 3. The VIN is visible here even though the grid's VIN toggle is off - the modal always shows it.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.9, §9), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.9, §9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5515,8 +5512,8 @@
 4. This is where whole-order vs subset scope is spelled out (the grid block only says 'N Lines').
 Note for the tester: the absence of any money figure is CORRECT and is what this test expects. The product owner ruled on 22 July 2026 that no total in dollars is shown anywhere on the Schedule. If you see no money figure, pass this test.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.9, §4.4), read on 11 August 2026. Version 23 of that specification asked for the lines to carry 'labor/total figures'. Version 25, published on 6 August 2026, changed that to 'labor/status figures', so the specification and this test now agree that no money figure is shown; the specification still asks for a labor figure, which this test does not expect, and on that one point the behaviour above follows the product owner's later decision of 22 July 2026, recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.9, §4.4), read on 17 August 2026. Version 23 of that specification asked for the lines to carry 'labor/total figures'. Version 25, published on 6 August 2026, changed that to 'labor/status figures', so the specification and this test now agree that no money figure is shown; the specification still asks for a labor figure, which this test does not expect, and on that one point the behaviour above follows the product owner's later decision of 22 July 2026, recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5568,8 +5565,8 @@
 2. The new value persists after closing and re-opening.
 3. Dependent displays (progress vs estimate) reflect the new value.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.9), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5584,7 +5581,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Notes can be added, edited, and deleted per work order from the modal</t>
+          <t>Notes can be added, edited, and deleted per shift from the modal</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -5620,16 +5617,16 @@
           <t xml:space="preserve">1. The note is added and shown in the modal.
 2. The edit is saved and displayed.
 3. The delete removes the note.
-4. Notes are kept per work order (the same note is visible from another shift of the same work order).
----
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.9), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: HOLD - not re-checked against the current build - it needs a drag that could not be completed
+4. Notes are kept per shift - a note added to one shift is shown on that shift only, not on other shifts of the same work order.
+---
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>SV-8695 (§4.9 (Notes: add,edit,and delete per work order))</t>
+          <t>SV-8695 (§4.9 (Notes: add/edit/delete per shift))</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -5677,8 +5674,8 @@
 3. 'Adjust' leads to a way to resolve the conflict (for example changing the shift's time).
 4. An unconflicted shift's modal shows no such banner.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.9), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5730,8 +5727,8 @@
 2. There is no 'Reassign' action in the modal; reassignment is done by dragging a shift to another technician row (covered by its own case).
 3. Delete on a series member asks for a deletion scope (the full scope behavior has its own cases).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.9, §7), read on 11 August 2026. That specification describes this point in two different ways, so the behaviour above follows its first-release wording and a product owner decision is still awaited; the open question is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.9, §7), read on 17 August 2026. That specification describes this point in two different ways, so the behaviour above follows its first-release wording and a product owner decision is still awaited; the open question is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5893,8 +5890,8 @@
 3. Saving creates an event block on that technician's day.
 4. A toast with Undo appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10, §7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10, §7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -5946,8 +5943,8 @@
 2. A live preview block is shown while creating, and dragging resizes it.
 3. Completing creates the event at the previewed time/duration.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6002,8 +5999,8 @@
 4. With all-day ON, specific start/end times are not required (the time fields are disabled or hidden).
 5. The event is created as an all-day block for that technician and day.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10, §8.1), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10, §8.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6056,8 +6053,8 @@
 2. Dropping on another day moves it to that day.
 3. Each move produces a toast with Undo.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10, §7), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: HOLD - not re-checked against the current build - it needs a drag that could not be completed
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10, §7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6108,8 +6105,8 @@
 2. It has a small grey-filled rounded chip on the left containing a calendar icon, and two lines of text beside it: the event name, then the time range in secondary text.
 3. The shift reads as a tinted color-filled block with a colored left rail - the two types are separable at a glance, not by color alone.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6162,8 +6159,8 @@
 2. The color picker offers the same custom color palette as shifts (shared picker with editable labels).
 3. Choosing a color tints the card and the icon chip in matching tones, the same way a colored shift is tinted.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10, §10), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10, §10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6216,8 +6213,8 @@
 2. The event does NOT create a double-booked or overlap conflict with the shift, and the toolbar conflict count does not increase because of it.
 3. The two behave differently on purpose: an event uses up capacity, but it is never flagged as a conflict.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.10, §4.11, §4.12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8696 and the Schedule specification version 30 (§4.10, §4.11, §4.12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6271,8 +6268,8 @@
 3. The toolbar conflict pill's count increases.
 4. The conflict is listed in the pill's dropdown.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.11), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8697 and the Schedule specification version 30 (§4.11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6437,8 +6434,8 @@
 3. The list covers all current conflicts (count matches the pill).
 4. Resolving a conflict (for example moving the shift) reduces the count - detection is continuous.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.11, §6), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8697 and the Schedule specification version 30 (§4.11, §6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6489,8 +6486,8 @@
           <t xml:space="preserve">1. The grid navigates to the relevant technician and day.
 2. The conflicted shift is brought into view.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.11), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8697 and the Schedule specification version 30 (§4.11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6541,8 +6538,8 @@
           <t xml:space="preserve">1. Overtime is signaled with the 'OT' text tag and amber tones - NOT red or alarming styling.
 2. Red/alarming styling appears only for conflicts and genuine errors.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.11, §4.12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8697 and the Schedule specification version 30 (§4.11, §4.12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6653,8 +6650,8 @@
 2. A more heavily booked day shows a longer blue fill; the fill never exceeds the track (clamped at 100%).
 3. The track width is identical across all days (capacity is not rescaled per day), so bars are comparable at a glance.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8698 and the Schedule specification version 30 (§4.12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6704,8 +6701,8 @@
           <t xml:space="preserve">1. An amber segment extends past the right edge of the track, showing the excess.
 2. A tick marks the 100% line where the track ends.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.12), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8698 and the Schedule specification version 30 (§4.12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6756,8 +6753,8 @@
 2. The tag is text, not a color-only signal.
 3. Overtime (per-technician) and capacity (aggregate) are independent signals.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.12, §11), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8698 and the Schedule specification version 30 (§4.12, §11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6920,10 +6917,10 @@
           <t xml:space="preserve">1. The tooltip shows: the customer name; unit, vehicle, and VIN (the tooltip shows the VIN whenever the unit has one, regardless of the 'VIN Number' toggle); the date and time range; the technician; and a scope summary ('N lines · Xh' style).
 2. The individual line names appear as a short list capped at 3, with a '+N more lines' row for the rest (here '+2 more lines'); line statuses are NOT shown.
 3. A time-logged progress bar shows logged vs estimated hours ('X / Yh' style).
-Known issue on the build tested: The tooltip listed ALL FIVE line names on the 5-line series shift with no "+N more lines" row. Spec 4.13: "the individual line names as a short list capped at 3 with a '+N more lines' row". Everything else matched: customer, unit and VIN, date and time range, technician, scope summary "5 lines - 12h" and the progress bar. VIN appears with the toggle off, per Branko 2026-07-31. It has been reported to the QA lead but has no developer ticket yet. Mark this test FAILED and note it in your run comment; do not raise a new ticket without asking the QA lead.
----
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.13), read on 11 August 2026. The behaviour above follows a later product owner decision dated 31 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+Known issue on the build tested: the tooltip shows the VIN only when the 'VIN Number' toggle inside 'Filter &amp; display' is switched ON. With that toggle OFF the tooltip shows the unit on its own (for example 'G30'); with it ON the same tooltip reads 'G30 - VIN 12-06696'. The expected behaviour above asks for the VIN whenever the unit has one, whichever way the toggle is set. It has been
+---
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.13), read on 17 August 2026. The behaviour above follows a later product owner decision dated 31 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -6973,8 +6970,8 @@
           <t xml:space="preserve">1. The customer name line includes the conflict icon.
 2. The conflict reason is shown in amber.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.13), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.13), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7025,8 +7022,8 @@
 2. The date and time range are shown.
 3. The technician is shown.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.13), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.13), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7081,8 +7078,8 @@
 3. The tooltip is read-only (no buttons/actions inside it).
 4. Clicking the block opens the full detail modal as normal.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.13), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.13), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7134,8 +7131,8 @@
 2. Near a side edge, the tooltip shifts horizontally to stay fully within the viewport.
 3. No part of the tooltip is clipped off-screen.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.13), read on 11 August 2026. Last checked against build v3.5-d122eef on 8/5/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§4.13), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7484,8 +7481,8 @@
           <t xml:space="preserve">1. The grid jumps to the range containing the current date (today's day, this week, or this month depending on the active view).
 2. The date label updates accordingly.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§6), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7538,8 +7535,8 @@
 3. Month view: each click moves one month; the label shows that month.
 4. The label always matches what the grid displays.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§6), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§6), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7591,10 +7588,9 @@
 2. All five of these are matched against, so searching any one of them finds the blocks it belongs to: customer name, work order number, unit number, technician name, and line name.
 3. Note for the tester: the specification does not say what happens to the blocks that do NOT match - whether they stay on the grid faded out, or disappear until you clear the search. Do not pass or fail this test on that. Check only that searching each of the five things above finds the right blocks. What happens to the non-matching blocks is an open question with the product owner.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§6, Search), read on 11 August 2026, which describes the search as filtering the grid blocks by matching against customer name, WO number, unit number, technician name, and line name.
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§6, Search), read on 17 August 2026, which describes the search as filtering the grid blocks by matching against customer name, WO number, unit number, technician name, and line name.
 This case used to also expect matching blocks to highlight and non-matching blocks to fade. That sentence was in version 23 of the specification; version 24, published on 6 August 2026, deleted it, and it has not come back in versions 25, 26 or 27. Story SV-8686 does still ask for it, but that wording has not been touched since the story was created on 27 July 2026, so the specification's deletion is the newer decision and it is the one this case now follows.
-Last checked against build v3.5-7ec992f on 8/6/2026; the wording above was corrected on 11 August 2026 from the documents only, with no build opened.
-AUTOMATION: READY
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7645,8 +7641,8 @@
 2. Defaults: all department toggles ON, 'My Shifts' OFF, 'VIN Number' OFF.
 3. There is no separate departments-only control - this dropdown replaces it.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§6, §9), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§6, §9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7699,8 +7695,8 @@
 2. Other departments are unaffected.
 3. Turning it back on restores the group.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§9), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7754,8 +7750,8 @@
 3. This is a personal convenience filter only - it does not change what you are permitted to see (default is OFF, everyone's shifts visible).
 4. For a user who has no technician/staff record of their own, the 'My Shifts' option is not shown at all.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§9, §14.3), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a user with no staff record of their own
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§9, §14.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7812,8 +7808,8 @@
 5. The 'VIN Number' toggle affects the block only - the tooltip and the modal always show the VIN when the unit has one.
 Note for the tester: the VIN staying visible in the hover summary and in the shift window while the VIN switch is off is CORRECT and is what this test expects. The product owner ruled on 31 July 2026 that the VIN is always visible on hover regardless of the switch. If you see it there, pass this test.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§9, §4.4, §4.8), read on 11 August 2026. The behaviour above follows a later product owner decision dated 31 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and stories SV-8700 and SV-8690 and SV-8694 and the Schedule specification version 30 (§9, §4.4, §4.8), read on 17 August 2026. The behaviour above follows a later product owner decision dated 31 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7868,8 +7864,8 @@
 3. Capacity Planning OFF: the capacity bars disappear from the column headers; ON: they reappear with the same values.
 4. Events OFF: event blocks disappear from the grid while shifts remain; ON: the events reappear unchanged.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§6, §9, §4.12), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§6, §9, §4.12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7922,8 +7918,8 @@
 2. Working hours remain unshaded.
 3. Turning it off removes the shading.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§9, §4.8), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§9, §4.8), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -7975,8 +7971,8 @@
 2. The hours match the technicians' configured hours.
 3. Turning it off hides the hours again.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§9), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§9), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8028,8 +8024,8 @@
 2. 'Show Sunday' off too: 5 weekday columns remain (Monday to Friday).
 3. Both back on: the full Monday-to-Sunday 7-column week returns.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§9, §3.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§9, §3.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8083,8 +8079,8 @@
 3. Technician B is added to the affected line's roster and technician A is removed from it.
 4. A toast with Undo appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7, §12), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8695 and the Schedule specification version 30 (§7, §12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8189,8 +8185,8 @@
           <t xml:space="preserve">1. The menu offers a 'New Work Order' item.
 2. Choosing it directs the user to create a work order (a toast / prompt pointing to the Work Orders tab).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7, §4.10), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§7, §4.10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8247,8 +8243,8 @@
 3. After you confirm, the block sits in the new technician's row, that technician is added to the work order line's technician list, and the previous one is taken off it.
 Why this test covers Week view only: the specification describes reassignment as dragging a shift from one technician row to another, and Month view has no technician rows at all - it is a calendar of day boxes. Whether reassignment should be possible in Month view is therefore part of the open question on SV-8867 and is deliberately not asserted here.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7, §12), read on 11 August 2026: dragging a shift block from one technician row to another reassigns it and a confirmation handles cross-technician moves, and a series is a grouping over ordinary daily shifts rather than a different kind of thing, so an ordinary shift's behaviour applies to a series member too. Story SV-8692 covers series-aware deletion only and says nothing about reassignment. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8867 and the Schedule specification version 30 (§7, §12), read on 17 August 2026: dragging a shift block from one technician row to another reassigns it and a confirmation handles cross-technician moves, and a series is a grouping over ordinary daily shifts rather than a different kind of thing, so an ordinary shift's behaviour applies to a series member too. Story SV-8692 covers series-aware deletion only and says nothing about reassignment.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8354,11 +8350,11 @@
       <c r="G145" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. A scope prompt appears with three options: this shift only, this and everything after, and the whole series.
-2. Each option states its consequence in hours returned (spec's example format: 'returns 8h' / 'returns 56h').
+2. Each option states how many scheduled hours it removes.
 3. The prompt uses routine, lightweight styling - not alarming destructive styling.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8400,7 +8396,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>1. Delete a middle shift with the 'this shift only' scope.
+          <t>1. Delete a middle shift with the 'This shift only' scope.
 2. Look at the series on the grid.
 3. Check the scheduled hours.</t>
         </is>
@@ -8409,11 +8405,11 @@
         <is>
           <t xml:space="preserve">1. Only that day's shift is removed.
 2. The series keeps the gap - the remaining shifts do NOT shuffle to close it.
-3. The removed day's hours return to the estimate's remaining (scheduled hours drop by that day's hours).
+3. The scheduled hours drop by that day's hours (the estimate and any clocked hours are separate quantities and are not changed by the deletion).
 4. An undo toast appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8455,7 +8451,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>1. Delete the series' THIRD shift with the 'this and everything after' scope.
+          <t>1. Delete the series' THIRD shift with the 'This and all later shifts' scope.
 2. Look at the series on the grid.</t>
         </is>
       </c>
@@ -8465,8 +8461,8 @@
 2. The first two shifts remain untouched.
 3. An undo toast appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8518,8 +8514,8 @@
 2. Technician B's independent series is untouched (the scope is per technician's series).
 3. An undo toast appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8573,8 +8569,8 @@
 3. Middle shift: all three options.
 4. Cancelling leaves the series unchanged in every case.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8625,8 +8621,8 @@
           <t xml:space="preserve">1. No series-scope prompt appears (the scope question is only for shifts that belong to a series).
 2. The shift is deleted and an undo toast appears.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8692 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8641,7 +8637,7 @@
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>Toast lasts ~7s with Undo (about 4s without); stays on hover, goes on leave</t>
+          <t>Toast stays 4 to 7 seconds, stays while hovered, goes when the cursor leaves</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -8674,12 +8670,12 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. Untouched, a toast that has an Undo action persists about 7 seconds; a toast without Undo persists about 4 seconds, before dismissing.
+          <t xml:space="preserve">1. Untouched, the toast stays on screen for between 4 and 7 seconds and then disappears on its own.
 2. While the cursor is over it, the toast stays (does not auto-dismiss).
 3. After the cursor leaves, it dismisses.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7, §11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§7, §11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8736,8 +8732,8 @@
 4. Undo after reassign: the shift returns to the original technician, and the line's roster is restored (original tech back on, target tech off).
 5. Every destructive action is undoable within the toast's lifetime.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7, §11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§7, §11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8792,8 +8788,8 @@
 3. Clicking Undo within the toast's lifetime reverses the action (the deleted shift comes back).
 4. Note for the tester: Undo works by performing a reversing action, not by holding the change back - a change surviving a refresh before Undo is expected, not a bug.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026, which requires the toast and its Undo. That specification does not say how Undo works underneath, so the point above - that the action is already saved and Undo reverses it rather than holding it back - comes from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8688 and the Schedule specification version 30 (§7), read on 17 August 2026, which requires the toast and its Undo. That specification does not say how Undo works underneath, so the point above - that the action is already saved and Undo reverses it rather than holding it back - comes from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8848,8 +8844,8 @@
 4. With two layers open, the FIRST Escape closes only the topmost layer, and the SECOND Escape closes the next layer down.
 5. Escape works anywhere on the schedule page as a global shortcut, following the defined stacking order (delete scope, reassign, spread, capacity, event modal, event view, line picker, shift detail, cell menu, calendar picker, customize, filters, search).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8905,8 +8901,8 @@
 3. In the note editor, Enter inserts a new line in the note - it does NOT confirm or close the dialog.
 4. The multiline note can be completed and saved normally.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§7), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§7), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -8958,8 +8954,8 @@
 2. Focus stays trapped inside the modal (wraps back to its first control) until the modal closes.
 3. On the page, toolbar and sidebar controls are reachable by keyboard.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9010,8 +9006,8 @@
           <t xml:space="preserve">1. Both the single shift and the multi-week series render in the default blue.
 2. No special color is auto-applied to long jobs - blue is the default for ALL shifts.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§10), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9066,8 +9062,8 @@
 3. The color is per SHIFT, not per work order - the other shift from the same work order keeps its own (default blue) color and does not change.
 4. Colors carry no fixed meaning - they are free choice beyond the two defaults (blue shift / grey event).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§10, §4.9, §4.4), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and stories SV-8700 and SV-8690 and the Schedule specification version 30 (§10, §4.9, §4.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9120,8 +9116,8 @@
 2. The renamed label shows for the whole shop - the same picker opened elsewhere shows 'ZZAUTOTEST Rush'.
 3. Shifts and events share the same custom palette with the same labels.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§10, §4.10), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8700 and the Schedule specification version 30 (§10, §4.10), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9177,8 +9173,8 @@
 4. Each day has a From time and a To time you can set.
 5. The saved shop business hours are used by the Schedule (start-time hierarchy, before/after-hours conflicts, business-hours shading).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8699 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9230,8 +9226,8 @@
 2. The toggle is OFF by default (no custom hours set).
 3. Turning it ON reveals a per-day working-hours editor for that technician.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8699 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9281,8 +9277,8 @@
           <t xml:space="preserve">1. With no custom hours, the technician's working hours fall back to the shop business hours.
 2. Start-time defaults and before/after-hours conflict checks for that technician use the shop business hours.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8699 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9333,8 +9329,8 @@
 2. The added range starts empty (no From/To pre-filled).
 3. Each added range can be removed individually.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8699 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9388,8 +9384,8 @@
 4. The incomplete row (empty From/To) is ignored by the overlap check - it does not raise the overlap error.
 5. Save is not blocked by an incomplete row on its own (only genuine overlaps disable Save).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8699 and the Schedule specification version 30 (§4.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9444,8 +9440,8 @@
 3. ALL technicians' shifts and events are visible (not just the user's own).
 4. Tooltips show on hover, and the shift/event detail modals open in read-only mode.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1, §14.3), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a view-only user
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1, §14.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9500,8 +9496,8 @@
 3. No creation menu opens at all - there is no 'Create Event' and no 'New Work Order' offered.
 4. In the modal, edit fields are hidden or disabled, and the reassign and delete actions are absent.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a view-only user
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9551,8 +9547,8 @@
           <t xml:space="preserve">1. The Schedule top-level nav item is not shown at all.
 2. The rest of the app works normally for the role.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a user without the Schedule permission
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9608,8 +9604,8 @@
 4. Edge-resize and horizontal drag work in day view.
 5. Modal fields are editable and save.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as an edit-without-delete user
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9662,8 +9658,8 @@
 2. Events likewise offer no delete.
 3. No path exists to remove shifts or events - while creating and modifying still work.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as an edit-without-delete user
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9717,8 +9713,8 @@
 3. Events can be deleted too.
 4. Undo toasts appear (restore the items via Undo to clean up).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a delete-capable user
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9770,8 +9766,8 @@
 2. Delete cannot be granted without Edit.
 3. The three tiers can be enabled in dependency order, so each higher level always includes the ones beneath it (Delete includes Edit, and Edit includes View).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9824,8 +9820,8 @@
 2. Shifts already on the grid can still be viewed and interacted with per the role's Schedule tier.
 3. New work orders cannot be dragged on - the WO list is simply not visible.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.2), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a user who cannot see work orders
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§14.2), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9876,8 +9872,8 @@
           <t xml:space="preserve">1. The user sees ALL technicians' shifts and events, not only their own - there is no role-based 'own shifts only' restriction.
 2. 'My Shifts' exists only as an optional personal convenience filter (off by default), not a security boundary.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.3), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a view-only technician
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.3), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9928,8 +9924,8 @@
           <t xml:space="preserve">1. The department-assigned staff member appears as a technician row - row presence is controlled by the department on the staff record, NOT by role permission.
 2. The staff member without a department does not appear as a row.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.4), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§14.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -9979,8 +9975,8 @@
           <t xml:space="preserve">1. The Time-Clock-ON staff member can clock in.
 2. The Time-Clock-OFF staff member cannot - the ability is controlled by the staff-record setting, not by the Schedule permission tier.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.4), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: HOLD - needs a second sign-in as each of the two staff members
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§14.4), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10033,8 +10029,8 @@
 2. The schedule structure itself (the shift's day, time, and technician) stays visible so the grid remains usable.
 3. This extends the sidebar behavior (the work order list and drill-down are hidden) to the work-order data surfaced on the shifts themselves.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.2), read on 11 August 2026. The behaviour above follows a later product owner decision dated 22 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a user who cannot see work orders
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§14.2), read on 17 August 2026. The behaviour above follows a later product owner decision dated 22 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10091,8 +10087,8 @@
 3. The user from step 4 gets the read-only schedule - nothing can be dragged onto the grid and no shift can be created.
 4. The user from step 5 can drag a work order onto the grid and create a shift.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14.1), read on 11 August 2026. Last checked against build v3.5-65d6500 on 8/12/2026.
-AUTOMATION: HOLD - needs a second sign-in as a holder of each permission level
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14.1), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10145,8 +10141,8 @@
 3. On narrow viewports the sidebar collapses.
 4. No content becomes permanently unreachable and nothing errors.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and stories SV-8686 and SV-8687 and the Schedule specification version 30 (§11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10199,8 +10195,8 @@
 2. The drill-down behaves the same with many lines.
 3. Search stays responsive on the long list.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the Schedule specification version 30 (§11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10253,8 +10249,8 @@
 2. View switches complete without long hangs.
 3. Tooltips and modals stay responsive.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8686 and the Schedule specification version 30 (§11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10358,8 +10354,8 @@
           <t xml:space="preserve">1. All three quantities are shown/derivable and may differ from one another.
 2. Nothing forces them to match - no error, no auto-correction (progress is driven by clocked-in time).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5, §12), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5, §12), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10410,8 +10406,8 @@
           <t xml:space="preserve">1. Every shift in the series starts at the SAME local wall-clock time (e.g. 8:00 AM) on both sides of the clock change.
 2. No shift in the series silently moves an hour earlier or later after the change date.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5), read on 11 August 2026, which covers spreading work across days. That specification says nothing about clock changes or daylight saving - those words do not appear in it at all - so the point above comes from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5), read on 17 August 2026, which covers spreading work across days. That specification says nothing about clock changes or daylight saving - those words do not appear in it at all - so the point above comes from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10465,8 +10461,8 @@
 3. Conflict and overtime cues remain distinguishable (they never rely on colour alone - text/icon still present).
 4. Switching back to light mode restores the normal look with nothing stuck in dark colours.
 ---
-This is the expected behaviour as per story SV-8700 (dark theme), read on 11 August 2026, story SV-8698 (overtime and conflict cues are not colour-only), read on 11 August 2026, and the Schedule specification version 27 (§11), read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per story SV-8700 (dark theme), read on 17 August 2026, story SV-8698 (overtime and conflict cues are not colour-only), read on 17 August 2026, and the Schedule specification version 30 (§11), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10528,8 +10524,8 @@
 4. At step 8, on the other computer or in the private window, the Schedule is ALSO in dark mode. The choice is remembered against your account, not against the one browser you set it in.
 5. Switching back to light mode at step 9 works the same way and is remembered in the same way.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, its story SV-8700 (requirement 5), read on 11 August 2026, and the Schedule specification version 27 (§11 Dark theme), read on 11 August 2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, its story SV-8700 (requirement 5), read on 17 August 2026, and the Schedule specification version 30 (§11 Dark theme), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10585,8 +10581,8 @@
 3. None of the three blends into the page so that its edges cannot be made out, and none of them is missing that separation entirely while the light-mode version has it.
 4. Nothing you check is unreadable, and no text or icon disappears into the background.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, its story SV-8700 (requirement 5), read on 11 August 2026, and the Schedule specification version 27 (§11 Dark theme), read on 11 August 2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, its story SV-8700 (requirement 5), read on 17 August 2026, and the Schedule specification version 30 (§11 Dark theme), read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10693,8 +10689,8 @@
 2. Events are still events and shifts are still shifts (nothing changed kind or vanished).
 3. Their details open normally and are editable/deletable like any other entry.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. No numbered requirement in the Schedule specification version 27 covers this point. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - cannot be run now - it needs shifts noted BEFORE the release, and the release is already deployed
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026. No numbered requirement in the Schedule specification version 30 covers this point.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10746,8 +10742,8 @@
 2. Note for the tester: before this release the Dashboard duplicated such a work order once per scheduled day - showing one combined row now is the intended fix, do not report it as a missing-rows bug.
 3. Work orders with a single shift are unaffected.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. No numbered requirement in the Schedule specification version 27 covers this point. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - the Dashboard section this test needs does not exist in the build
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026. No numbered requirement in the Schedule specification version 30 covers this point.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10799,8 +10795,8 @@
 2. It behaves like any other scheduled entry (opens, moves, deletes normally).
 3. It also appears in the Dashboard's schedule section for that day.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. No numbered requirement in the Schedule specification version 27 covers this point. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - work order creation offers no appointment in the build
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026. No numbered requirement in the Schedule specification version 30 covers this point.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10853,8 +10849,8 @@
 2. The shift does NOT appear on location B's board, even though the technician is enrolled there too.
 3. Note for the tester: before the rewrite such a shift showed on EVERY location the technician was enrolled at - showing it only on the work order's location is the intended new behaviour, do not report the disappearance from other locations as a bug.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. No numbered requirement in the Schedule specification version 27 covers this point. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026. No numbered requirement in the Schedule specification version 30 covers this point.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10908,8 +10904,8 @@
 3. After saving, the Schedule sidebar reflects the chosen priority and the Priority filter finds the work order under High.
 4. A work order with no priority set simply shows none (it is not treated as an error).
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. No numbered requirement in the Schedule specification version 27 covers this point. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - the Priority field this test needs does not exist in the build
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8687 and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026. No numbered requirement in the Schedule specification version 30 covers this point.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -10963,8 +10959,8 @@
 3. View + Edit: the POST and PATCH succeed (HTTP 201/200); the DELETE is refused with HTTP 403 because the user lacks Schedule: Delete.
 4. Each refusal is a clean 403 response - never a server error.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14), read on 11 August 2026, which sets the three permission levels. That specification does not describe what the server returns when a request is refused, so the refusal responses above come from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs three separate sign-ins, one per permission level
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14), read on 17 August 2026, which sets the three permission levels. That specification does not describe what the server returns when a request is refused, so the refusal responses above come from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -11018,8 +11014,8 @@
 3. The over-120-shift request is refused with HTTP 422 even WITH the acknowledgement - the hard cap cannot be overridden.
 4. Refused calls leave no partial series behind.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§4.5), read on 11 August 2026, with the specific limits above taken from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and story SV-8691 and the Schedule specification version 30 (§4.5), read on 17 August 2026, with the specific limits above taken from the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -11071,8 +11067,8 @@
 2. For the caller without Work Orders: View, the work-order-derived details (customer, unit, VIN, line names) are absent/empty in the response itself - not just hidden on screen.
 3. Both calls still succeed (HTTP 200) - lacking Work Orders: View limits the content, it does not break the schedule read.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the Schedule specification version 27 (§14), read on 11 August 2026. The behaviour above follows a later product owner decision dated 22 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 11 August 2026. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: HOLD - needs a second sign-in as a user who cannot see work orders
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the Schedule specification version 30 (§14), read on 17 August 2026. The behaviour above follows a later product owner decision dated 22 July 2026 rather than that specification's wording, and that decision is recorded in Branko's answers, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/branko-answers-2026-07-31/answers-ingested.md, read on 17 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>
@@ -11115,7 +11111,7 @@
       <c r="F196" s="2" t="inlineStr">
         <is>
           <t>1. While scoped to location A, call GET /api/schedule/shifts/{id} with the location-B shift id.
-2. Also try PATCH /api/schedule/shifts/{id} on the same id.
+2. Also try PATCH /api/schedule/shifts/{id} on the same id, changing a real field such as the colour. (A request that would change nothing is rejected on its own account before the location is even checked, so always send a real change here.)
 3. Call GET /api/schedule/board for location A's current week.</t>
         </is>
       </c>
@@ -11125,8 +11121,8 @@
 2. The PATCH on the foreign id is refused the same way (404) - no cross-location edit is possible.
 3. Location A's board contains only location A's shifts - nothing from location B leaks in.
 ---
-This is the expected behaviour as per epic SV-8685, read on 11 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 11 August 2026. No numbered requirement in the Schedule specification version 27 covers this point. Last checked against build v3.5-7ec992f on 8/6/2026.
-AUTOMATION: READY
+This is the expected behaviour as per epic SV-8685, read on 17 August 2026, and the engineering technical plan, in this file: https://github.com/bilalmuzamil-sketch/Manual-test-Cases/blob/HEAD/build/schedule/tech-plan-2026-07-29/TechPlan-Schedule-Module-Rewrite.md, read on 17 August 2026. No numbered requirement in the Schedule specification version 30 covers this point.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/17/2026
 </t>
         </is>
       </c>

</xml_diff>